<commit_message>
Daily ratings update: 2026-08-06
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -848,10 +848,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>223909</v>
+        <v>223908</v>
       </c>
       <c r="C2" t="n">
-        <v>4.696083</v>
+        <v>4.696131</v>
       </c>
       <c r="F2" t="n">
         <v>320219</v>
@@ -1150,10 +1150,10 @@
         <v>1000000</v>
       </c>
       <c r="R2" t="n">
-        <v>4.696083</v>
+        <v>4.696131</v>
       </c>
       <c r="T2" t="n">
-        <v>223909</v>
+        <v>223908</v>
       </c>
       <c r="U2" t="n">
         <v>17118</v>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-07
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2</f>
+              <f>'Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2</f>
+              <f>'Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2</f>
+              <f>'Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2</f>
+              <f>'Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2</f>
+              <f>'Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2</f>
+              <f>'Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2</f>
+              <f>'Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2</f>
+              <f>'Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -860,6 +860,37 @@
         <v>4.73752</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>224046</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.696341</v>
+      </c>
+      <c r="D3" t="n">
+        <v>121</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.189</v>
+      </c>
+      <c r="F3" t="n">
+        <v>320406</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.73758</v>
+      </c>
+      <c r="H3" t="n">
+        <v>187</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -872,7 +903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1201,6 +1232,142 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.696341</v>
+      </c>
+      <c r="T3" t="n">
+        <v>224046</v>
+      </c>
+      <c r="U3" t="n">
+        <v>17122</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1212,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1373,6 +1540,76 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.73758</v>
+      </c>
+      <c r="E3" t="n">
+        <v>320406</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.73758</v>
+      </c>
+      <c r="G3" t="n">
+        <v>320406</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-08
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$3</f>
+              <f>'Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$3</f>
+              <f>'Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$3</f>
+              <f>'Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$3</f>
+              <f>'Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$3</f>
+              <f>'Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$3</f>
+              <f>'Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$3</f>
+              <f>'Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$3</f>
+              <f>'Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -891,6 +891,37 @@
         <v>4.84</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>224189</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.6962247</v>
+      </c>
+      <c r="D4" t="n">
+        <v>143</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.514</v>
+      </c>
+      <c r="F4" t="n">
+        <v>320593</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.73761</v>
+      </c>
+      <c r="H4" t="n">
+        <v>187</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.789</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -903,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1368,6 +1399,142 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.6962247</v>
+      </c>
+      <c r="T4" t="n">
+        <v>224189</v>
+      </c>
+      <c r="U4" t="n">
+        <v>17126</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1379,7 +1546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1610,6 +1777,76 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.73761</v>
+      </c>
+      <c r="E4" t="n">
+        <v>320593</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.73761</v>
+      </c>
+      <c r="G4" t="n">
+        <v>320593</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-09
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$4</f>
+              <f>'Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$4</f>
+              <f>'Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$4</f>
+              <f>'Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$4</f>
+              <f>'Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$4</f>
+              <f>'Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -922,6 +922,37 @@
         <v>4.789</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>224324</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.6965303</v>
+      </c>
+      <c r="D5" t="n">
+        <v>135</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.204</v>
+      </c>
+      <c r="F5" t="n">
+        <v>320734</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="H5" t="n">
+        <v>141</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -934,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1535,6 +1566,142 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.6965303</v>
+      </c>
+      <c r="T5" t="n">
+        <v>224324</v>
+      </c>
+      <c r="U5" t="n">
+        <v>17134</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1546,7 +1713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1847,6 +2014,76 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="E5" t="n">
+        <v>320734</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="G5" t="n">
+        <v>320734</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-10
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$5</f>
+              <f>'Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$5</f>
+              <f>'Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$5</f>
+              <f>'Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$5</f>
+              <f>'Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$5</f>
+              <f>'Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$5</f>
+              <f>'Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$5</f>
+              <f>'Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$5</f>
+              <f>'Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -953,6 +953,34 @@
         <v>4.578</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>224434</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.695349</v>
+      </c>
+      <c r="D6" t="n">
+        <v>110</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.286</v>
+      </c>
+      <c r="F6" t="n">
+        <v>320679</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-55</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -965,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1702,6 +1730,142 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.695349</v>
+      </c>
+      <c r="T6" t="n">
+        <v>224434</v>
+      </c>
+      <c r="U6" t="n">
+        <v>17138</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1713,7 +1877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2084,6 +2248,76 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="E6" t="n">
+        <v>320679</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="G6" t="n">
+        <v>320679</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-11
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$6</f>
+              <f>'Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$6</f>
+              <f>'Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$6</f>
+              <f>'Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$6</f>
+              <f>'Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$6</f>
+              <f>'Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$6</f>
+              <f>'Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$6</f>
+              <f>'Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$6</f>
+              <f>'Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -981,6 +981,37 @@
         <v>-55</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>224568</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.6959743</v>
+      </c>
+      <c r="D7" t="n">
+        <v>134</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.743</v>
+      </c>
+      <c r="F7" t="n">
+        <v>320757</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="H7" t="n">
+        <v>78</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.738</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -993,7 +1024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1866,6 +1897,142 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.6959743</v>
+      </c>
+      <c r="T7" t="n">
+        <v>224568</v>
+      </c>
+      <c r="U7" t="n">
+        <v>17146</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1877,7 +2044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2318,6 +2485,76 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="E7" t="n">
+        <v>320757</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.73754</v>
+      </c>
+      <c r="G7" t="n">
+        <v>320757</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-12
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$7</f>
+              <f>'Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$7</f>
+              <f>'Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$7</f>
+              <f>'Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$7</f>
+              <f>'Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$7</f>
+              <f>'Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$7</f>
+              <f>'Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$7</f>
+              <f>'Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$7</f>
+              <f>'Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1012,6 +1012,37 @@
         <v>4.738</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>224742</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.697012</v>
+      </c>
+      <c r="D8" t="n">
+        <v>174</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6.036</v>
+      </c>
+      <c r="F8" t="n">
+        <v>320936</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.73747</v>
+      </c>
+      <c r="H8" t="n">
+        <v>179</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.612</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1024,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2033,6 +2064,142 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.697012</v>
+      </c>
+      <c r="T8" t="n">
+        <v>224742</v>
+      </c>
+      <c r="U8" t="n">
+        <v>17153</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2044,7 +2211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2555,6 +2722,76 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.73747</v>
+      </c>
+      <c r="E8" t="n">
+        <v>320936</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.73747</v>
+      </c>
+      <c r="G8" t="n">
+        <v>320936</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-13
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$8</f>
+              <f>'Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$8</f>
+              <f>'Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$8</f>
+              <f>'Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$8</f>
+              <f>'Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$8</f>
+              <f>'Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$8</f>
+              <f>'Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$8</f>
+              <f>'Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$8</f>
+              <f>'Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,37 @@
         <v>4.612</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>224873</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.697567</v>
+      </c>
+      <c r="D9" t="n">
+        <v>131</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F9" t="n">
+        <v>321107</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.7374</v>
+      </c>
+      <c r="H9" t="n">
+        <v>171</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.606</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1055,7 +1086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2200,6 +2231,142 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.697567</v>
+      </c>
+      <c r="T9" t="n">
+        <v>224873</v>
+      </c>
+      <c r="U9" t="n">
+        <v>17162</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2211,7 +2378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2792,6 +2959,76 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.7374</v>
+      </c>
+      <c r="E9" t="n">
+        <v>321107</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.7374</v>
+      </c>
+      <c r="G9" t="n">
+        <v>321107</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-14
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$9</f>
+              <f>'Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$9</f>
+              <f>'Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$9</f>
+              <f>'Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$9</f>
+              <f>'Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$9</f>
+              <f>'Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$9</f>
+              <f>'Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$9</f>
+              <f>'Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$9</f>
+              <f>'Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1074,6 +1074,37 @@
         <v>4.606</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>225021</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.697548</v>
+      </c>
+      <c r="D10" t="n">
+        <v>148</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.669</v>
+      </c>
+      <c r="F10" t="n">
+        <v>321302</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.73736</v>
+      </c>
+      <c r="H10" t="n">
+        <v>195</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.671</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1086,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2367,6 +2398,142 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.697548</v>
+      </c>
+      <c r="T10" t="n">
+        <v>225021</v>
+      </c>
+      <c r="U10" t="n">
+        <v>17165</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2378,7 +2545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3029,6 +3196,76 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.73736</v>
+      </c>
+      <c r="E10" t="n">
+        <v>321302</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.73736</v>
+      </c>
+      <c r="G10" t="n">
+        <v>321302</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-15
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$10</f>
+              <f>'Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$10</f>
+              <f>'Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$10</f>
+              <f>'Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$10</f>
+              <f>'Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$10</f>
+              <f>'Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$10</f>
+              <f>'Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$10</f>
+              <f>'Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$10</f>
+              <f>'Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1105,6 +1105,37 @@
         <v>4.671</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>225134</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.697199</v>
+      </c>
+      <c r="D11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.002</v>
+      </c>
+      <c r="F11" t="n">
+        <v>321486</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.73739</v>
+      </c>
+      <c r="H11" t="n">
+        <v>184</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1117,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2534,6 +2565,142 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.697199</v>
+      </c>
+      <c r="T11" t="n">
+        <v>225134</v>
+      </c>
+      <c r="U11" t="n">
+        <v>17168</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2545,7 +2712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3266,6 +3433,76 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.73739</v>
+      </c>
+      <c r="E11" t="n">
+        <v>321486</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.73739</v>
+      </c>
+      <c r="G11" t="n">
+        <v>321486</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-16
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$11</f>
+              <f>'Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$11</f>
+              <f>'Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$11</f>
+              <f>'Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$11</f>
+              <f>'Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$11</f>
+              <f>'Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$11</f>
+              <f>'Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$11</f>
+              <f>'Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$11</f>
+              <f>'Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1136,6 +1136,37 @@
         <v>4.79</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>225137</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.696472</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-49.861</v>
+      </c>
+      <c r="F12" t="n">
+        <v>321514</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="H12" t="n">
+        <v>28</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.623</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1148,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2701,6 +2732,142 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.696472</v>
+      </c>
+      <c r="T12" t="n">
+        <v>225137</v>
+      </c>
+      <c r="U12" t="n">
+        <v>17170</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2712,7 +2879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3503,6 +3670,76 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="E12" t="n">
+        <v>321514</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="G12" t="n">
+        <v>321514</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-17
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$12</f>
+              <f>'Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$12</f>
+              <f>'Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$12</f>
+              <f>'Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$12</f>
+              <f>'Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$12</f>
+              <f>'Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$12</f>
+              <f>'Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$12</f>
+              <f>'Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$12</f>
+              <f>'Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1167,6 +1167,37 @@
         <v>4.623</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>225141</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.6965604</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9.672000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>321518</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="H13" t="n">
+        <v>4</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.737</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1179,7 +1210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2868,6 +2899,142 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>16.20.2</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1785273709</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.6965604</v>
+      </c>
+      <c r="T13" t="n">
+        <v>225141</v>
+      </c>
+      <c r="U13" t="n">
+        <v>17171</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/qSLLcrjyZXDLG6RpJH4LusumhpFEqRUFRE4Jl83jxJSrU-0JYUPRDkr0xmv2o0tzTkFd5G-VDScumlVfoGOYEA</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2879,7 +3046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3740,6 +3907,76 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="E13" t="n">
+        <v>321518</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.73738</v>
+      </c>
+      <c r="G13" t="n">
+        <v>321518</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>16.20.1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-07-28T15:22:00Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-18
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -185,12 +185,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$13</f>
+              <f>'Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$D$2:$D$13</f>
+              <f>'Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -217,12 +217,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$13</f>
+              <f>'Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$H$2:$H$13</f>
+              <f>'Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -336,12 +336,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$13</f>
+              <f>'Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$E$2:$E$13</f>
+              <f>'Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -368,12 +368,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Summary'!$A$2:$A$13</f>
+              <f>'Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Summary'!$I$2:$I$13</f>
+              <f>'Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1198,6 +1198,31 @@
         <v>4.737</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>225130</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.696751</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-11</v>
+      </c>
+      <c r="F14" t="n">
+        <v>321516</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.73737</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1210,7 +1235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3035,6 +3060,142 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.696751</v>
+      </c>
+      <c r="T14" t="n">
+        <v>225130</v>
+      </c>
+      <c r="U14" t="n">
+        <v>17173</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3046,7 +3207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3977,6 +4138,76 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.73737</v>
+      </c>
+      <c r="E14" t="n">
+        <v>321516</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.73737</v>
+      </c>
+      <c r="G14" t="n">
+        <v>321516</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-19
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$14</f>
+              <f>'ENBD Summary'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$14</f>
+              <f>'ENBD Summary'!$D$2:$D$15</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$14</f>
+              <f>'ENBD Summary'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$14</f>
+              <f>'ENBD Summary'!$H$2:$H$15</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2</f>
+              <f>'ADCB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2</f>
+              <f>'ADCB Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2</f>
+              <f>'ADCB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2</f>
+              <f>'ADCB Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2</f>
+              <f>'ADIB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2</f>
+              <f>'ADIB Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2</f>
+              <f>'ADIB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2</f>
+              <f>'ADIB Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2</f>
+              <f>'ADIB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2</f>
+              <f>'ADIB Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2</f>
+              <f>'ADIB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2</f>
+              <f>'ADIB Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2</f>
+              <f>'FAB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2</f>
+              <f>'FAB Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2</f>
+              <f>'FAB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2</f>
+              <f>'FAB Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2</f>
+              <f>'FAB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2</f>
+              <f>'FAB Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2</f>
+              <f>'FAB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2</f>
+              <f>'FAB Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2</f>
+              <f>'RAK Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2</f>
+              <f>'RAK Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2</f>
+              <f>'RAK Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2</f>
+              <f>'RAK Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2</f>
+              <f>'RAK Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2</f>
+              <f>'RAK Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2</f>
+              <f>'RAK Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2</f>
+              <f>'RAK Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$14</f>
+              <f>'ENBD Summary'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$14</f>
+              <f>'ENBD Summary'!$E$2:$E$15</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$14</f>
+              <f>'ENBD Summary'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$14</f>
+              <f>'ENBD Summary'!$I$2:$I$15</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2</f>
+              <f>'EI Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2</f>
+              <f>'EI Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2</f>
+              <f>'EI Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2</f>
+              <f>'EI Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2</f>
+              <f>'EI Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2</f>
+              <f>'EI Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2</f>
+              <f>'EI Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2</f>
+              <f>'EI Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2</f>
+              <f>'MASHREQ Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2</f>
+              <f>'MASHREQ Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2</f>
+              <f>'MASHREQ Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2</f>
+              <f>'MASHREQ Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2</f>
+              <f>'MASHREQ Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2</f>
+              <f>'MASHREQ Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2</f>
+              <f>'MASHREQ Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2</f>
+              <f>'MASHREQ Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2</f>
+              <f>'WIO Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2</f>
+              <f>'WIO Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2</f>
+              <f>'WIO Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2</f>
+              <f>'WIO Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2</f>
+              <f>'WIO Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2</f>
+              <f>'WIO Summary'!$E$2:$E$3</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2</f>
+              <f>'WIO Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2</f>
+              <f>'WIO Summary'!$I$2:$I$3</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2</f>
+              <f>'ADCB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2</f>
+              <f>'ADCB Summary'!$D$2:$D$3</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2</f>
+              <f>'ADCB Summary'!$A$2:$A$3</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2</f>
+              <f>'ADCB Summary'!$H$2:$H$3</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4055,6 +4055,31 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>225124</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4.696885</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F15" t="n">
+        <v>321512</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4.73733</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4067,7 +4092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4147,6 +4172,37 @@
         <v>4.80866</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5751</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.6090426</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>83.629</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6652</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.80818</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4159,7 +4215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4495,6 +4551,149 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.6090426</v>
+      </c>
+      <c r="T3" t="n">
+        <v>5751</v>
+      </c>
+      <c r="U3" t="n">
+        <v>519</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4506,7 +4705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4675,6 +4874,84 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.80818</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6652</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80818</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6652</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4686,7 +4963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4766,6 +5043,31 @@
         <v>4.68151</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>64338</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.218525</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>113017</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4778,7 +5080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5114,6 +5416,149 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.218525</v>
+      </c>
+      <c r="T3" t="n">
+        <v>64338</v>
+      </c>
+      <c r="U3" t="n">
+        <v>15249</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5125,7 +5570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5295,6 +5740,85 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="E3" t="n">
+        <v>113017</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="G3" t="n">
+        <v>113017</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5306,7 +5830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5386,6 +5910,37 @@
         <v>4.47058</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>72649</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.692165</v>
+      </c>
+      <c r="D3" t="n">
+        <v>149</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6.503</v>
+      </c>
+      <c r="F3" t="n">
+        <v>73813</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.47091</v>
+      </c>
+      <c r="H3" t="n">
+        <v>203</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.591</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5398,7 +5953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5737,6 +6292,152 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1784679266</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.692165</v>
+      </c>
+      <c r="T3" t="n">
+        <v>72649</v>
+      </c>
+      <c r="U3" t="n">
+        <v>4789</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5748,7 +6449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5920,6 +6621,87 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.47091</v>
+      </c>
+      <c r="E3" t="n">
+        <v>73813</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.47091</v>
+      </c>
+      <c r="G3" t="n">
+        <v>73813</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-04T21:10:14Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5931,7 +6713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6011,6 +6793,37 @@
         <v>4.70263</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>45320</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.633374</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.575</v>
+      </c>
+      <c r="F3" t="n">
+        <v>251705</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.70266</v>
+      </c>
+      <c r="H3" t="n">
+        <v>51</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.851</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6023,7 +6836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AE15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7984,6 +8797,142 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R15" t="n">
+        <v>4.696885</v>
+      </c>
+      <c r="T15" t="n">
+        <v>225124</v>
+      </c>
+      <c r="U15" t="n">
+        <v>17177</v>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W15" t="b">
+        <v>1</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7995,7 +8944,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8345,6 +9294,163 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.633374</v>
+      </c>
+      <c r="T3" t="n">
+        <v>45320</v>
+      </c>
+      <c r="U3" t="n">
+        <v>15009</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8356,7 +9462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8535,6 +9641,94 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.70266</v>
+      </c>
+      <c r="E3" t="n">
+        <v>251705</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.70266</v>
+      </c>
+      <c r="G3" t="n">
+        <v>251705</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8546,7 +9740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8626,6 +9820,37 @@
         <v>4.63472</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>43776</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.308777</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-9.94</v>
+      </c>
+      <c r="F3" t="n">
+        <v>111028</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.63469</v>
+      </c>
+      <c r="H3" t="n">
+        <v>53</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.572</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8638,7 +9863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8983,6 +10208,158 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>3.7.67</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1787030060</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.308777</v>
+      </c>
+      <c r="T3" t="n">
+        <v>43776</v>
+      </c>
+      <c r="U3" t="n">
+        <v>12340</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8994,7 +10371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9172,6 +10549,93 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.63469</v>
+      </c>
+      <c r="E3" t="n">
+        <v>111028</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.63469</v>
+      </c>
+      <c r="G3" t="n">
+        <v>111028</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2.0.92</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:10:13Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9183,7 +10647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9263,6 +10727,37 @@
         <v>4.63544</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>46134</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.4835196</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-45.763</v>
+      </c>
+      <c r="F3" t="n">
+        <v>33711</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.6353</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.849</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9275,7 +10770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9612,6 +11107,150 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>350.55.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1786843173</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.4835196</v>
+      </c>
+      <c r="T3" t="n">
+        <v>46134</v>
+      </c>
+      <c r="U3" t="n">
+        <v>3260</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9623,7 +11262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9793,6 +11432,85 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.6353</v>
+      </c>
+      <c r="E3" t="n">
+        <v>33711</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.6353</v>
+      </c>
+      <c r="G3" t="n">
+        <v>33711</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-17T05:24:07Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9804,7 +11522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10805,6 +12523,76 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4.73733</v>
+      </c>
+      <c r="E15" t="n">
+        <v>321512</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.73733</v>
+      </c>
+      <c r="G15" t="n">
+        <v>321512</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10816,7 +12604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10896,6 +12684,34 @@
         <v>4.71784</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>73786</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.674979</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>113659</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.71774</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.965</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10908,7 +12724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11229,6 +13045,134 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.674979</v>
+      </c>
+      <c r="T3" t="n">
+        <v>73786</v>
+      </c>
+      <c r="U3" t="n">
+        <v>5907</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11240,7 +13184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11395,6 +13339,70 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.71774</v>
+      </c>
+      <c r="E3" t="n">
+        <v>113659</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.71774</v>
+      </c>
+      <c r="G3" t="n">
+        <v>113659</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11406,7 +13414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11486,6 +13494,37 @@
         <v>4.80385</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>141797</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4.756382</v>
+      </c>
+      <c r="D3" t="n">
+        <v>161</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.738</v>
+      </c>
+      <c r="F3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="H3" t="n">
+        <v>112</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4.596</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11498,7 +13537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11861,167 +13900,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -12067,6 +13967,420 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R3" t="n">
+        <v>4.756382</v>
+      </c>
+      <c r="T3" t="n">
+        <v>141797</v>
+      </c>
+      <c r="U3" t="n">
+        <v>11000</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-20
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$15</f>
+              <f>'ENBD Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$15</f>
+              <f>'ENBD Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$15</f>
+              <f>'ENBD Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$15</f>
+              <f>'ENBD Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$3</f>
+              <f>'ADCB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$3</f>
+              <f>'ADCB Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$3</f>
+              <f>'ADCB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$3</f>
+              <f>'ADCB Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$3</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$3</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$3</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$3</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$3</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$3</f>
+              <f>'ADIB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$3</f>
+              <f>'ADIB Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$3</f>
+              <f>'ADIB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$3</f>
+              <f>'ADIB Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$3</f>
+              <f>'ADIB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$3</f>
+              <f>'ADIB Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$3</f>
+              <f>'ADIB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$3</f>
+              <f>'ADIB Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$3</f>
+              <f>'FAB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$3</f>
+              <f>'FAB Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$3</f>
+              <f>'FAB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$3</f>
+              <f>'FAB Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$3</f>
+              <f>'FAB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$3</f>
+              <f>'FAB Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$3</f>
+              <f>'FAB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$3</f>
+              <f>'FAB Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$3</f>
+              <f>'RAK Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$3</f>
+              <f>'RAK Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$3</f>
+              <f>'RAK Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$3</f>
+              <f>'RAK Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$3</f>
+              <f>'RAK Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$3</f>
+              <f>'RAK Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$3</f>
+              <f>'RAK Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$3</f>
+              <f>'RAK Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$15</f>
+              <f>'ENBD Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$15</f>
+              <f>'ENBD Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$15</f>
+              <f>'ENBD Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$15</f>
+              <f>'ENBD Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$3</f>
+              <f>'EI Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$3</f>
+              <f>'EI Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$3</f>
+              <f>'EI Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$3</f>
+              <f>'EI Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$3</f>
+              <f>'EI Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$3</f>
+              <f>'EI Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$3</f>
+              <f>'EI Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$3</f>
+              <f>'EI Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$3</f>
+              <f>'MASHREQ Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$3</f>
+              <f>'MASHREQ Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$3</f>
+              <f>'MASHREQ Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$3</f>
+              <f>'MASHREQ Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$3</f>
+              <f>'MASHREQ Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$3</f>
+              <f>'MASHREQ Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$3</f>
+              <f>'MASHREQ Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$3</f>
+              <f>'MASHREQ Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$3</f>
+              <f>'WIO Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$3</f>
+              <f>'WIO Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$3</f>
+              <f>'WIO Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$3</f>
+              <f>'WIO Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$3</f>
+              <f>'WIO Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$3</f>
+              <f>'WIO Summary'!$E$2:$E$4</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$3</f>
+              <f>'WIO Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$3</f>
+              <f>'WIO Summary'!$I$2:$I$4</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$3</f>
+              <f>'ADCB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$3</f>
+              <f>'ADCB Summary'!$D$2:$D$4</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$3</f>
+              <f>'ADCB Summary'!$A$2:$A$4</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$3</f>
+              <f>'ADCB Summary'!$H$2:$H$4</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4080,6 +4080,37 @@
         <v>-4</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>225136</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.696259</v>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-7.048</v>
+      </c>
+      <c r="F16" t="n">
+        <v>321518</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.7373</v>
+      </c>
+      <c r="H16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4092,7 +4123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4203,6 +4234,37 @@
         <v>4.01</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5755</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.600529</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-7.64</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6658</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.8082</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.83</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4215,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4694,6 +4756,149 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.600529</v>
+      </c>
+      <c r="T4" t="n">
+        <v>5755</v>
+      </c>
+      <c r="U4" t="n">
+        <v>519</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4705,7 +4910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4952,6 +5157,84 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.8082</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6658</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.8082</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6658</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4963,7 +5246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5068,6 +5351,31 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>64337</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.2186904</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>113016</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5080,7 +5388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5559,6 +5867,149 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.2186904</v>
+      </c>
+      <c r="T4" t="n">
+        <v>64337</v>
+      </c>
+      <c r="U4" t="n">
+        <v>15248</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5570,7 +6021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5819,6 +6270,85 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="E4" t="n">
+        <v>113016</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="G4" t="n">
+        <v>113016</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5830,7 +6360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5941,6 +6471,37 @@
         <v>4.591</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>72834</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.6928234</v>
+      </c>
+      <c r="D4" t="n">
+        <v>185</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.951</v>
+      </c>
+      <c r="F4" t="n">
+        <v>73994</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.47146</v>
+      </c>
+      <c r="H4" t="n">
+        <v>181</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.696</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5953,7 +6514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6438,6 +6999,152 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1784679266</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.6928234</v>
+      </c>
+      <c r="T4" t="n">
+        <v>72834</v>
+      </c>
+      <c r="U4" t="n">
+        <v>4796</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6449,7 +7156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6702,6 +7409,87 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.47146</v>
+      </c>
+      <c r="E4" t="n">
+        <v>73994</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.47146</v>
+      </c>
+      <c r="G4" t="n">
+        <v>73994</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-04T21:10:14Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6713,7 +7501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6824,6 +7612,37 @@
         <v>4.851</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>45333</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.634625</v>
+      </c>
+      <c r="D4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E4" t="n">
+        <v>8.996</v>
+      </c>
+      <c r="F4" t="n">
+        <v>251764</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.70272</v>
+      </c>
+      <c r="H4" t="n">
+        <v>59</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.959</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6836,7 +7655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8933,6 +9752,142 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.696259</v>
+      </c>
+      <c r="T16" t="n">
+        <v>225136</v>
+      </c>
+      <c r="U16" t="n">
+        <v>17182</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8944,7 +9899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9451,6 +10406,163 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.634625</v>
+      </c>
+      <c r="T4" t="n">
+        <v>45333</v>
+      </c>
+      <c r="U4" t="n">
+        <v>15012</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9462,7 +10574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9729,6 +10841,94 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.70272</v>
+      </c>
+      <c r="E4" t="n">
+        <v>251764</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.70272</v>
+      </c>
+      <c r="G4" t="n">
+        <v>251764</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9740,7 +10940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9851,6 +11051,37 @@
         <v>4.572</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>43790</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.3103843</v>
+      </c>
+      <c r="D4" t="n">
+        <v>14</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9.336</v>
+      </c>
+      <c r="F4" t="n">
+        <v>111073</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="H4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.709</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9863,7 +11094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10360,6 +11591,158 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>3.7.67</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1787030060</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.3103843</v>
+      </c>
+      <c r="T4" t="n">
+        <v>43790</v>
+      </c>
+      <c r="U4" t="n">
+        <v>12344</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10371,7 +11754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10636,6 +12019,93 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="E4" t="n">
+        <v>111073</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="G4" t="n">
+        <v>111073</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.0.92</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:10:13Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10647,7 +12117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10758,6 +12228,37 @@
         <v>3.849</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.4822874</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-2.624</v>
+      </c>
+      <c r="F4" t="n">
+        <v>33712</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.63526</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3.287</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10770,7 +12271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11251,6 +12752,150 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>350.55.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1786843173</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.4822874</v>
+      </c>
+      <c r="T4" t="n">
+        <v>46142</v>
+      </c>
+      <c r="U4" t="n">
+        <v>3260</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11262,7 +12907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11511,6 +13156,85 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.63526</v>
+      </c>
+      <c r="E4" t="n">
+        <v>33712</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.63526</v>
+      </c>
+      <c r="G4" t="n">
+        <v>33712</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-17T05:24:07Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11522,7 +13246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12593,6 +14317,76 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.7373</v>
+      </c>
+      <c r="E16" t="n">
+        <v>321518</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.7373</v>
+      </c>
+      <c r="G16" t="n">
+        <v>321518</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12604,7 +14398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12712,6 +14506,34 @@
         <v>-0.965</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>73810</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.676049</v>
+      </c>
+      <c r="D4" t="n">
+        <v>24</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7.966</v>
+      </c>
+      <c r="F4" t="n">
+        <v>113658</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.71764</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12724,7 +14546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13173,6 +14995,134 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.676049</v>
+      </c>
+      <c r="T4" t="n">
+        <v>73810</v>
+      </c>
+      <c r="U4" t="n">
+        <v>5911</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13184,7 +15134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13403,6 +15353,70 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.71764</v>
+      </c>
+      <c r="E4" t="n">
+        <v>113658</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.71764</v>
+      </c>
+      <c r="G4" t="n">
+        <v>113658</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13414,7 +15428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13525,6 +15539,37 @@
         <v>4.596</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>142110</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.757271</v>
+      </c>
+      <c r="D4" t="n">
+        <v>313</v>
+      </c>
+      <c r="E4" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="F4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="H4" t="n">
+        <v>94</v>
+      </c>
+      <c r="I4" t="n">
+        <v>4.862</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13537,7 +15582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14070,167 +16115,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -14276,66 +16182,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R4" t="n">
+        <v>4.757271</v>
+      </c>
+      <c r="T4" t="n">
+        <v>142110</v>
+      </c>
+      <c r="U4" t="n">
+        <v>11013</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -14382,6 +16492,216 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-21
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$16</f>
+              <f>'ENBD Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$16</f>
+              <f>'ENBD Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$16</f>
+              <f>'ENBD Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$16</f>
+              <f>'ENBD Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$4</f>
+              <f>'ADCB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$4</f>
+              <f>'ADCB Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$4</f>
+              <f>'ADCB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$4</f>
+              <f>'ADCB Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$4</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$4</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$4</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$4</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$4</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$4</f>
+              <f>'ADIB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$4</f>
+              <f>'ADIB Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$4</f>
+              <f>'ADIB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$4</f>
+              <f>'ADIB Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$4</f>
+              <f>'ADIB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$4</f>
+              <f>'ADIB Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$4</f>
+              <f>'ADIB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$4</f>
+              <f>'ADIB Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$4</f>
+              <f>'FAB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$4</f>
+              <f>'FAB Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$4</f>
+              <f>'FAB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$4</f>
+              <f>'FAB Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$4</f>
+              <f>'FAB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$4</f>
+              <f>'FAB Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$4</f>
+              <f>'FAB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$4</f>
+              <f>'FAB Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$4</f>
+              <f>'RAK Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$4</f>
+              <f>'RAK Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$4</f>
+              <f>'RAK Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$4</f>
+              <f>'RAK Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$4</f>
+              <f>'RAK Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$4</f>
+              <f>'RAK Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$4</f>
+              <f>'RAK Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$4</f>
+              <f>'RAK Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$16</f>
+              <f>'ENBD Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$16</f>
+              <f>'ENBD Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$16</f>
+              <f>'ENBD Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$16</f>
+              <f>'ENBD Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$4</f>
+              <f>'EI Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$4</f>
+              <f>'EI Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$4</f>
+              <f>'EI Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$4</f>
+              <f>'EI Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$4</f>
+              <f>'EI Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$4</f>
+              <f>'EI Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$4</f>
+              <f>'EI Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$4</f>
+              <f>'EI Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$4</f>
+              <f>'MASHREQ Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$4</f>
+              <f>'MASHREQ Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$4</f>
+              <f>'MASHREQ Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$4</f>
+              <f>'MASHREQ Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$4</f>
+              <f>'MASHREQ Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$4</f>
+              <f>'MASHREQ Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$4</f>
+              <f>'MASHREQ Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$4</f>
+              <f>'MASHREQ Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$4</f>
+              <f>'WIO Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$4</f>
+              <f>'WIO Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$4</f>
+              <f>'WIO Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$4</f>
+              <f>'WIO Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$4</f>
+              <f>'WIO Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$4</f>
+              <f>'WIO Summary'!$E$2:$E$5</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$4</f>
+              <f>'WIO Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$4</f>
+              <f>'WIO Summary'!$I$2:$I$5</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$4</f>
+              <f>'ADCB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$4</f>
+              <f>'ADCB Summary'!$D$2:$D$5</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$4</f>
+              <f>'ADCB Summary'!$A$2:$A$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$4</f>
+              <f>'ADCB Summary'!$H$2:$H$5</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4111,6 +4111,34 @@
         <v>3.13</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>225142</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.6946383</v>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-56.118</v>
+      </c>
+      <c r="F17" t="n">
+        <v>321516</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.73725</v>
+      </c>
+      <c r="H17" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4123,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4265,6 +4293,37 @@
         <v>4.83</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5759</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.6147757</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25.112</v>
+      </c>
+      <c r="F5" t="n">
+        <v>6664</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.80792</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.497</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4277,7 +4336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4899,6 +4958,149 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.6147757</v>
+      </c>
+      <c r="T5" t="n">
+        <v>5759</v>
+      </c>
+      <c r="U5" t="n">
+        <v>520</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4910,7 +5112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5235,6 +5437,84 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.80792</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6664</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80792</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6664</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5246,7 +5526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5376,6 +5656,34 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64339</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.2184324</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-4.081</v>
+      </c>
+      <c r="F5" t="n">
+        <v>113010</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5388,7 +5696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6010,6 +6318,149 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.2184324</v>
+      </c>
+      <c r="T5" t="n">
+        <v>64339</v>
+      </c>
+      <c r="U5" t="n">
+        <v>15248</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6021,7 +6472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6349,6 +6800,85 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="E5" t="n">
+        <v>113010</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="G5" t="n">
+        <v>113010</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6360,7 +6890,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6502,6 +7032,37 @@
         <v>4.696</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>73001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.693953</v>
+      </c>
+      <c r="D5" t="n">
+        <v>167</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.187</v>
+      </c>
+      <c r="F5" t="n">
+        <v>74174</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.47172</v>
+      </c>
+      <c r="H5" t="n">
+        <v>180</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.579</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6514,7 +7075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7145,6 +7706,152 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.693953</v>
+      </c>
+      <c r="T5" t="n">
+        <v>73001</v>
+      </c>
+      <c r="U5" t="n">
+        <v>4803</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7156,7 +7863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7490,6 +8197,87 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.47172</v>
+      </c>
+      <c r="E5" t="n">
+        <v>74174</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.47172</v>
+      </c>
+      <c r="G5" t="n">
+        <v>74174</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7501,7 +8289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7643,6 +8431,37 @@
         <v>4.959</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>45337</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.634983</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>8.692</v>
+      </c>
+      <c r="F5" t="n">
+        <v>251819</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.70253</v>
+      </c>
+      <c r="H5" t="n">
+        <v>55</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.833</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7655,7 +8474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9888,6 +10707,142 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.6946383</v>
+      </c>
+      <c r="T17" t="n">
+        <v>225142</v>
+      </c>
+      <c r="U17" t="n">
+        <v>17179</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9899,7 +10854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10563,6 +11518,163 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.634983</v>
+      </c>
+      <c r="T5" t="n">
+        <v>45337</v>
+      </c>
+      <c r="U5" t="n">
+        <v>15015</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10574,7 +11686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10929,6 +12041,94 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.70253</v>
+      </c>
+      <c r="E5" t="n">
+        <v>251819</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.70253</v>
+      </c>
+      <c r="G5" t="n">
+        <v>251819</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10940,7 +12140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11082,6 +12282,37 @@
         <v>4.709</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>43799</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.3097496</v>
+      </c>
+      <c r="D5" t="n">
+        <v>9</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.222</v>
+      </c>
+      <c r="F5" t="n">
+        <v>111134</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.63486</v>
+      </c>
+      <c r="H5" t="n">
+        <v>61</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11094,7 +12325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11743,6 +12974,158 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>3.7.67</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1787030060</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.3097496</v>
+      </c>
+      <c r="T5" t="n">
+        <v>43799</v>
+      </c>
+      <c r="U5" t="n">
+        <v>12346</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11754,7 +13137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12106,6 +13489,93 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.63486</v>
+      </c>
+      <c r="E5" t="n">
+        <v>111134</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.63486</v>
+      </c>
+      <c r="G5" t="n">
+        <v>111134</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2.0.92</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:10:13Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12117,7 +13587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12259,6 +13729,37 @@
         <v>3.287</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>46144</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.4822974</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.713</v>
+      </c>
+      <c r="F5" t="n">
+        <v>33715</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.736</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12271,7 +13772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12896,6 +14397,150 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>350.55.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1786843173</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.4822974</v>
+      </c>
+      <c r="T5" t="n">
+        <v>46144</v>
+      </c>
+      <c r="U5" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12907,7 +14552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13235,6 +14880,85 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="E5" t="n">
+        <v>33715</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="G5" t="n">
+        <v>33715</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-17T05:24:07Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13246,7 +14970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14387,6 +16111,76 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.73725</v>
+      </c>
+      <c r="E17" t="n">
+        <v>321516</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.73725</v>
+      </c>
+      <c r="G17" t="n">
+        <v>321516</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14398,7 +16192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14534,6 +16328,37 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>73822</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.675711</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.597</v>
+      </c>
+      <c r="F5" t="n">
+        <v>113664</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.339</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -14546,7 +16371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15123,6 +16948,134 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.675711</v>
+      </c>
+      <c r="T5" t="n">
+        <v>73822</v>
+      </c>
+      <c r="U5" t="n">
+        <v>5911</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15134,7 +17087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15417,6 +17370,70 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="E5" t="n">
+        <v>113664</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="G5" t="n">
+        <v>113664</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15428,7 +17445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15570,6 +17587,37 @@
         <v>4.862</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>142384</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4.760092</v>
+      </c>
+      <c r="D5" t="n">
+        <v>274</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6.223</v>
+      </c>
+      <c r="F5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="H5" t="n">
+        <v>111</v>
+      </c>
+      <c r="I5" t="n">
+        <v>4.631</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -15582,7 +17630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE4"/>
+  <dimension ref="A1:AE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16285,167 +18333,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -16491,66 +18400,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R5" t="n">
+        <v>4.760092</v>
+      </c>
+      <c r="T5" t="n">
+        <v>142384</v>
+      </c>
+      <c r="U5" t="n">
+        <v>11023</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -16597,65 +18710,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -16702,6 +18815,216 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-22
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$17</f>
+              <f>'ENBD Summary'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$17</f>
+              <f>'ENBD Summary'!$D$2:$D$18</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$17</f>
+              <f>'ENBD Summary'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$17</f>
+              <f>'ENBD Summary'!$H$2:$H$18</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$5</f>
+              <f>'ADCB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$5</f>
+              <f>'ADCB Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$5</f>
+              <f>'ADCB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$5</f>
+              <f>'ADCB Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$5</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$5</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$5</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$5</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$5</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$5</f>
+              <f>'ADIB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$5</f>
+              <f>'ADIB Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$5</f>
+              <f>'ADIB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$5</f>
+              <f>'ADIB Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$5</f>
+              <f>'ADIB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$5</f>
+              <f>'ADIB Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$5</f>
+              <f>'ADIB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$5</f>
+              <f>'ADIB Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$5</f>
+              <f>'FAB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$5</f>
+              <f>'FAB Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$5</f>
+              <f>'FAB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$5</f>
+              <f>'FAB Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$5</f>
+              <f>'FAB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$5</f>
+              <f>'FAB Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$5</f>
+              <f>'FAB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$5</f>
+              <f>'FAB Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$5</f>
+              <f>'RAK Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$5</f>
+              <f>'RAK Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$5</f>
+              <f>'RAK Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$5</f>
+              <f>'RAK Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$5</f>
+              <f>'RAK Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$5</f>
+              <f>'RAK Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$5</f>
+              <f>'RAK Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$5</f>
+              <f>'RAK Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$17</f>
+              <f>'ENBD Summary'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$17</f>
+              <f>'ENBD Summary'!$E$2:$E$18</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$17</f>
+              <f>'ENBD Summary'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$17</f>
+              <f>'ENBD Summary'!$I$2:$I$18</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$5</f>
+              <f>'EI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$5</f>
+              <f>'EI Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$5</f>
+              <f>'EI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$5</f>
+              <f>'EI Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$5</f>
+              <f>'EI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$5</f>
+              <f>'EI Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$5</f>
+              <f>'EI Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$5</f>
+              <f>'EI Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$5</f>
+              <f>'MASHREQ Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$5</f>
+              <f>'MASHREQ Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$5</f>
+              <f>'MASHREQ Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$5</f>
+              <f>'MASHREQ Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$5</f>
+              <f>'MASHREQ Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$5</f>
+              <f>'MASHREQ Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$5</f>
+              <f>'MASHREQ Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$5</f>
+              <f>'MASHREQ Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$5</f>
+              <f>'WIO Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$5</f>
+              <f>'WIO Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$5</f>
+              <f>'WIO Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$5</f>
+              <f>'WIO Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$5</f>
+              <f>'WIO Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$5</f>
+              <f>'WIO Summary'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$5</f>
+              <f>'WIO Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$5</f>
+              <f>'WIO Summary'!$I$2:$I$6</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$5</f>
+              <f>'ADCB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$5</f>
+              <f>'ADCB Summary'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$5</f>
+              <f>'ADCB Summary'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$5</f>
+              <f>'ADCB Summary'!$H$2:$H$6</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4139,6 +4139,37 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>225157</v>
+      </c>
+      <c r="C18" t="n">
+        <v>4.6943893</v>
+      </c>
+      <c r="D18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="F18" t="n">
+        <v>321522</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.73724</v>
+      </c>
+      <c r="H18" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" t="n">
+        <v>4.201</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4151,7 +4182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4324,6 +4355,37 @@
         <v>4.497</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5765</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.6147757</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.615</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6671</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.80753</v>
+      </c>
+      <c r="H6" t="n">
+        <v>7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.436</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4336,7 +4398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5101,6 +5163,149 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.6147757</v>
+      </c>
+      <c r="T6" t="n">
+        <v>5765</v>
+      </c>
+      <c r="U6" t="n">
+        <v>521</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5112,7 +5317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5515,6 +5720,84 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.80753</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6671</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80753</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6671</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5526,7 +5809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5684,6 +5967,31 @@
         <v>-6</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>64338</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.2184324</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>113006</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -5696,7 +6004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6461,6 +6769,149 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.2184324</v>
+      </c>
+      <c r="T6" t="n">
+        <v>64338</v>
+      </c>
+      <c r="U6" t="n">
+        <v>15249</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6472,7 +6923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6879,6 +7330,85 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="E6" t="n">
+        <v>113006</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="G6" t="n">
+        <v>113006</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6890,7 +7420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7063,6 +7593,37 @@
         <v>4.579</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>73159</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.692724</v>
+      </c>
+      <c r="D6" t="n">
+        <v>158</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.125</v>
+      </c>
+      <c r="F6" t="n">
+        <v>74355</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.47197</v>
+      </c>
+      <c r="H6" t="n">
+        <v>181</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.574</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7075,7 +7636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7852,6 +8413,152 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.692724</v>
+      </c>
+      <c r="T6" t="n">
+        <v>73159</v>
+      </c>
+      <c r="U6" t="n">
+        <v>4813</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7863,7 +8570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8278,6 +8985,87 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.47197</v>
+      </c>
+      <c r="E6" t="n">
+        <v>74355</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.47197</v>
+      </c>
+      <c r="G6" t="n">
+        <v>74355</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8289,7 +9077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8462,6 +9250,37 @@
         <v>3.833</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>45341</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.63487</v>
+      </c>
+      <c r="D6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3.354</v>
+      </c>
+      <c r="F6" t="n">
+        <v>251866</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.70254</v>
+      </c>
+      <c r="H6" t="n">
+        <v>47</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.756</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8474,7 +9293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10843,6 +11662,142 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R18" t="n">
+        <v>4.6943893</v>
+      </c>
+      <c r="T18" t="n">
+        <v>225157</v>
+      </c>
+      <c r="U18" t="n">
+        <v>17178</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W18" t="b">
+        <v>1</v>
+      </c>
+      <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10854,7 +11809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11675,6 +12630,163 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.63487</v>
+      </c>
+      <c r="T6" t="n">
+        <v>45341</v>
+      </c>
+      <c r="U6" t="n">
+        <v>15018</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11686,7 +12798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12129,6 +13241,94 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.70254</v>
+      </c>
+      <c r="E6" t="n">
+        <v>251866</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.70254</v>
+      </c>
+      <c r="G6" t="n">
+        <v>251866</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12140,7 +13340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12313,6 +13513,37 @@
         <v>4.89</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>43807</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.307582</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-7.56</v>
+      </c>
+      <c r="F6" t="n">
+        <v>111176</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="H6" t="n">
+        <v>42</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.264</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12325,7 +13556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13126,6 +14357,158 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>3.7.67</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1787030060</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.307582</v>
+      </c>
+      <c r="T6" t="n">
+        <v>43807</v>
+      </c>
+      <c r="U6" t="n">
+        <v>12351</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13137,7 +14520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13576,6 +14959,93 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="E6" t="n">
+        <v>111176</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.63472</v>
+      </c>
+      <c r="G6" t="n">
+        <v>111176</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2.0.92</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:10:13Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13587,7 +15057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13760,6 +15230,31 @@
         <v>3.736</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.481182</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>33713</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13772,7 +15267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14541,6 +16036,150 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>350.55.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1786843173</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.481182</v>
+      </c>
+      <c r="T6" t="n">
+        <v>46143</v>
+      </c>
+      <c r="U6" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14552,7 +16191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14959,6 +16598,85 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="E6" t="n">
+        <v>33713</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="G6" t="n">
+        <v>33713</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-17T05:24:07Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14970,7 +16688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16181,6 +17899,76 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4.73724</v>
+      </c>
+      <c r="E18" t="n">
+        <v>321522</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4.73724</v>
+      </c>
+      <c r="G18" t="n">
+        <v>321522</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16192,7 +17980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16359,6 +18147,34 @@
         <v>4.339</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>73827</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.6753736</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-0.306</v>
+      </c>
+      <c r="F6" t="n">
+        <v>113661</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -16371,7 +18187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17076,6 +18892,134 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.6753736</v>
+      </c>
+      <c r="T6" t="n">
+        <v>73827</v>
+      </c>
+      <c r="U6" t="n">
+        <v>5912</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17087,7 +19031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17434,6 +19378,70 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="E6" t="n">
+        <v>113661</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="G6" t="n">
+        <v>113661</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17445,7 +19453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17618,6 +19626,37 @@
         <v>4.631</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>142546</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4.7574444</v>
+      </c>
+      <c r="D6" t="n">
+        <v>162</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="F6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="H6" t="n">
+        <v>92</v>
+      </c>
+      <c r="I6" t="n">
+        <v>4.565</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -17630,7 +19669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE5"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18503,167 +20542,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -18709,66 +20609,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R6" t="n">
+        <v>4.7574444</v>
+      </c>
+      <c r="T6" t="n">
+        <v>142546</v>
+      </c>
+      <c r="U6" t="n">
+        <v>11035</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -18815,65 +20919,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -18920,65 +21024,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -19025,6 +21129,216 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-23
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$18</f>
+              <f>'ENBD Summary'!$A$2:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$18</f>
+              <f>'ENBD Summary'!$D$2:$D$19</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$18</f>
+              <f>'ENBD Summary'!$A$2:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$18</f>
+              <f>'ENBD Summary'!$H$2:$H$19</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$6</f>
+              <f>'ADCB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$6</f>
+              <f>'ADCB Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$6</f>
+              <f>'ADCB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$6</f>
+              <f>'ADCB Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$6</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$6</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$6</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$6</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$6</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$6</f>
+              <f>'ADIB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$6</f>
+              <f>'ADIB Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$6</f>
+              <f>'ADIB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$6</f>
+              <f>'ADIB Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$6</f>
+              <f>'ADIB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$6</f>
+              <f>'ADIB Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$6</f>
+              <f>'ADIB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$6</f>
+              <f>'ADIB Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$6</f>
+              <f>'FAB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$6</f>
+              <f>'FAB Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$6</f>
+              <f>'FAB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$6</f>
+              <f>'FAB Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$6</f>
+              <f>'FAB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$6</f>
+              <f>'FAB Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$6</f>
+              <f>'FAB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$6</f>
+              <f>'FAB Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$6</f>
+              <f>'RAK Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$6</f>
+              <f>'RAK Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$6</f>
+              <f>'RAK Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$6</f>
+              <f>'RAK Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$6</f>
+              <f>'RAK Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$6</f>
+              <f>'RAK Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$6</f>
+              <f>'RAK Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$6</f>
+              <f>'RAK Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$18</f>
+              <f>'ENBD Summary'!$A$2:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$18</f>
+              <f>'ENBD Summary'!$E$2:$E$19</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$18</f>
+              <f>'ENBD Summary'!$A$2:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$18</f>
+              <f>'ENBD Summary'!$I$2:$I$19</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$6</f>
+              <f>'EI Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$6</f>
+              <f>'EI Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$6</f>
+              <f>'EI Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$6</f>
+              <f>'EI Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$6</f>
+              <f>'EI Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$6</f>
+              <f>'EI Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$6</f>
+              <f>'EI Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$6</f>
+              <f>'EI Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$6</f>
+              <f>'MASHREQ Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$6</f>
+              <f>'MASHREQ Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$6</f>
+              <f>'MASHREQ Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$6</f>
+              <f>'MASHREQ Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$6</f>
+              <f>'MASHREQ Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$6</f>
+              <f>'MASHREQ Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$6</f>
+              <f>'MASHREQ Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$6</f>
+              <f>'MASHREQ Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$6</f>
+              <f>'WIO Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$6</f>
+              <f>'WIO Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$6</f>
+              <f>'WIO Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$6</f>
+              <f>'WIO Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$6</f>
+              <f>'WIO Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$6</f>
+              <f>'WIO Summary'!$E$2:$E$7</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$6</f>
+              <f>'WIO Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$6</f>
+              <f>'WIO Summary'!$I$2:$I$7</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$6</f>
+              <f>'ADCB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$6</f>
+              <f>'ADCB Summary'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$6</f>
+              <f>'ADCB Summary'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$6</f>
+              <f>'ADCB Summary'!$H$2:$H$7</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4170,6 +4170,37 @@
         <v>4.201</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>225168</v>
+      </c>
+      <c r="C19" t="n">
+        <v>4.69428</v>
+      </c>
+      <c r="D19" t="n">
+        <v>11</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.457</v>
+      </c>
+      <c r="F19" t="n">
+        <v>321531</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4.73721</v>
+      </c>
+      <c r="H19" t="n">
+        <v>9</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3.665</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4182,7 +4213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4386,6 +4417,37 @@
         <v>4.436</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5773</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.6047745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-2.602</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6675</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.80764</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.991</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4398,7 +4460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5306,6 +5368,149 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.6047745</v>
+      </c>
+      <c r="T7" t="n">
+        <v>5773</v>
+      </c>
+      <c r="U7" t="n">
+        <v>522</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5317,7 +5522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5798,6 +6003,84 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.80764</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6675</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80764</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6675</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5809,7 +6092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5992,6 +6275,31 @@
         <v>-4</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>64319</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.218174</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-19</v>
+      </c>
+      <c r="F7" t="n">
+        <v>113006</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6004,7 +6312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6912,6 +7220,149 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.218174</v>
+      </c>
+      <c r="T7" t="n">
+        <v>64319</v>
+      </c>
+      <c r="U7" t="n">
+        <v>15246</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6923,7 +7374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7409,6 +7860,85 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="E7" t="n">
+        <v>113006</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.6815</v>
+      </c>
+      <c r="G7" t="n">
+        <v>113006</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7420,7 +7950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7624,6 +8154,37 @@
         <v>4.574</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>73321</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.6930037</v>
+      </c>
+      <c r="D7" t="n">
+        <v>162</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.819</v>
+      </c>
+      <c r="F7" t="n">
+        <v>74517</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.47219</v>
+      </c>
+      <c r="H7" t="n">
+        <v>162</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.573</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7636,7 +8197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8559,6 +9120,152 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.6930037</v>
+      </c>
+      <c r="T7" t="n">
+        <v>73321</v>
+      </c>
+      <c r="U7" t="n">
+        <v>4819</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8570,7 +9277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9066,6 +9773,87 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.47219</v>
+      </c>
+      <c r="E7" t="n">
+        <v>74517</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.47219</v>
+      </c>
+      <c r="G7" t="n">
+        <v>74517</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9077,7 +9865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9281,6 +10069,37 @@
         <v>4.756</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>45352</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.6372333</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14.379</v>
+      </c>
+      <c r="F7" t="n">
+        <v>251906</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.70248</v>
+      </c>
+      <c r="H7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.325</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9293,7 +10112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11798,6 +12617,142 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R19" t="n">
+        <v>4.69428</v>
+      </c>
+      <c r="T19" t="n">
+        <v>225168</v>
+      </c>
+      <c r="U19" t="n">
+        <v>17182</v>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W19" t="b">
+        <v>1</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11809,7 +12764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12787,6 +13742,163 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.6372333</v>
+      </c>
+      <c r="T7" t="n">
+        <v>45352</v>
+      </c>
+      <c r="U7" t="n">
+        <v>15022</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12798,7 +13910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13329,6 +14441,94 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.70248</v>
+      </c>
+      <c r="E7" t="n">
+        <v>251906</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.70248</v>
+      </c>
+      <c r="G7" t="n">
+        <v>251906</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13340,7 +14540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13544,6 +14744,37 @@
         <v>4.264</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>43819</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.306874</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="F7" t="n">
+        <v>111218</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="H7" t="n">
+        <v>42</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.926</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13556,7 +14787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14509,6 +15740,158 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>3.7.67</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1787030060</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.306874</v>
+      </c>
+      <c r="T7" t="n">
+        <v>43819</v>
+      </c>
+      <c r="U7" t="n">
+        <v>12356</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14520,7 +15903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15046,6 +16429,93 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="E7" t="n">
+        <v>111218</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="G7" t="n">
+        <v>111218</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2.0.92</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:10:13Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15057,7 +16527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15255,6 +16725,34 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.4816155</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11.149</v>
+      </c>
+      <c r="F7" t="n">
+        <v>33712</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -15267,7 +16765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16180,6 +17678,150 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>350.57.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1787428673</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.4816155</v>
+      </c>
+      <c r="T7" t="n">
+        <v>46146</v>
+      </c>
+      <c r="U7" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16191,7 +17833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16677,6 +18319,85 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="E7" t="n">
+        <v>33712</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="G7" t="n">
+        <v>33712</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:32:27Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16688,7 +18409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17969,6 +19690,76 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>4.73721</v>
+      </c>
+      <c r="E19" t="n">
+        <v>321531</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.73721</v>
+      </c>
+      <c r="G19" t="n">
+        <v>321531</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17980,7 +19771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18175,6 +19966,37 @@
         <v>-3</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>73828</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.6754804</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="F7" t="n">
+        <v>113664</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.718</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -18187,7 +20009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19020,6 +20842,134 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.6754804</v>
+      </c>
+      <c r="T7" t="n">
+        <v>73828</v>
+      </c>
+      <c r="U7" t="n">
+        <v>5912</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19031,7 +20981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19442,6 +21392,70 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="E7" t="n">
+        <v>113664</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="G7" t="n">
+        <v>113664</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19453,7 +21467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19657,6 +21671,37 @@
         <v>4.565</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>142733</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4.756459</v>
+      </c>
+      <c r="D7" t="n">
+        <v>187</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.005</v>
+      </c>
+      <c r="F7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="H7" t="n">
+        <v>91</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -19669,7 +21714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE6"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20712,167 +22757,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -20918,66 +22824,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R7" t="n">
+        <v>4.756459</v>
+      </c>
+      <c r="T7" t="n">
+        <v>142733</v>
+      </c>
+      <c r="U7" t="n">
+        <v>11050</v>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -21024,65 +23134,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -21129,65 +23239,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -21234,65 +23344,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -21339,6 +23449,216 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-24
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$19</f>
+              <f>'ENBD Summary'!$A$2:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$19</f>
+              <f>'ENBD Summary'!$D$2:$D$20</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$19</f>
+              <f>'ENBD Summary'!$A$2:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$19</f>
+              <f>'ENBD Summary'!$H$2:$H$20</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$7</f>
+              <f>'ADCB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$7</f>
+              <f>'ADCB Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$7</f>
+              <f>'ADCB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$7</f>
+              <f>'ADCB Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$7</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$7</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$7</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$7</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$7</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$7</f>
+              <f>'ADIB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$7</f>
+              <f>'ADIB Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$7</f>
+              <f>'ADIB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$7</f>
+              <f>'ADIB Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$7</f>
+              <f>'ADIB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$7</f>
+              <f>'ADIB Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$7</f>
+              <f>'ADIB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$7</f>
+              <f>'ADIB Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$7</f>
+              <f>'FAB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$7</f>
+              <f>'FAB Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$7</f>
+              <f>'FAB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$7</f>
+              <f>'FAB Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$7</f>
+              <f>'FAB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$7</f>
+              <f>'FAB Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$7</f>
+              <f>'FAB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$7</f>
+              <f>'FAB Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$7</f>
+              <f>'RAK Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$7</f>
+              <f>'RAK Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$7</f>
+              <f>'RAK Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$7</f>
+              <f>'RAK Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$7</f>
+              <f>'RAK Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$7</f>
+              <f>'RAK Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$7</f>
+              <f>'RAK Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$7</f>
+              <f>'RAK Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$19</f>
+              <f>'ENBD Summary'!$A$2:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$19</f>
+              <f>'ENBD Summary'!$E$2:$E$20</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$19</f>
+              <f>'ENBD Summary'!$A$2:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$19</f>
+              <f>'ENBD Summary'!$I$2:$I$20</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$7</f>
+              <f>'EI Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$7</f>
+              <f>'EI Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$7</f>
+              <f>'EI Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$7</f>
+              <f>'EI Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$7</f>
+              <f>'EI Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$7</f>
+              <f>'EI Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$7</f>
+              <f>'EI Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$7</f>
+              <f>'EI Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$7</f>
+              <f>'MASHREQ Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$7</f>
+              <f>'MASHREQ Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$7</f>
+              <f>'MASHREQ Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$7</f>
+              <f>'MASHREQ Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$7</f>
+              <f>'MASHREQ Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$7</f>
+              <f>'MASHREQ Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$7</f>
+              <f>'MASHREQ Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$7</f>
+              <f>'MASHREQ Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$7</f>
+              <f>'WIO Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$7</f>
+              <f>'WIO Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$7</f>
+              <f>'WIO Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$7</f>
+              <f>'WIO Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$7</f>
+              <f>'WIO Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$7</f>
+              <f>'WIO Summary'!$E$2:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$7</f>
+              <f>'WIO Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$7</f>
+              <f>'WIO Summary'!$I$2:$I$8</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$7</f>
+              <f>'ADCB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$7</f>
+              <f>'ADCB Summary'!$D$2:$D$8</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$7</f>
+              <f>'ADCB Summary'!$A$2:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$7</f>
+              <f>'ADCB Summary'!$H$2:$H$8</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4201,6 +4201,37 @@
         <v>3.665</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>225173</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4.6939144</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-11.77</v>
+      </c>
+      <c r="F20" t="n">
+        <v>321539</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4.73718</v>
+      </c>
+      <c r="H20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3.531</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4213,7 +4244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4448,6 +4479,37 @@
         <v>4.991</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5781</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.6062994</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.707</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6682</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.80783</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.989</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4460,7 +4522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5511,6 +5573,149 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.6062994</v>
+      </c>
+      <c r="T8" t="n">
+        <v>5781</v>
+      </c>
+      <c r="U8" t="n">
+        <v>523</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5522,7 +5727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6081,6 +6286,84 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.80783</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6682</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80783</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6682</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6092,7 +6375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6300,6 +6583,34 @@
         <v>0</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>64315</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.218174</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F8" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5.247</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6312,7 +6623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7363,6 +7674,149 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.218174</v>
+      </c>
+      <c r="T8" t="n">
+        <v>64315</v>
+      </c>
+      <c r="U8" t="n">
+        <v>15247</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7374,7 +7828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7939,6 +8393,85 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="E8" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.68151</v>
+      </c>
+      <c r="G8" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7950,7 +8483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8185,6 +8718,37 @@
         <v>4.573</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>73447</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.6932435</v>
+      </c>
+      <c r="D8" t="n">
+        <v>126</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.833</v>
+      </c>
+      <c r="F8" t="n">
+        <v>74704</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.4726</v>
+      </c>
+      <c r="H8" t="n">
+        <v>187</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.636</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8197,7 +8761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9266,6 +9830,152 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.6932435</v>
+      </c>
+      <c r="T8" t="n">
+        <v>73447</v>
+      </c>
+      <c r="U8" t="n">
+        <v>4834</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9277,7 +9987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9854,6 +10564,87 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.4726</v>
+      </c>
+      <c r="E8" t="n">
+        <v>74704</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.4726</v>
+      </c>
+      <c r="G8" t="n">
+        <v>74704</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9865,7 +10656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10100,6 +10891,37 @@
         <v>4.325</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>45357</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.636386</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-3.049</v>
+      </c>
+      <c r="F8" t="n">
+        <v>251976</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.70221</v>
+      </c>
+      <c r="H8" t="n">
+        <v>70</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3.731</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10112,7 +10934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:AE20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12753,6 +13575,142 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R20" t="n">
+        <v>4.6939144</v>
+      </c>
+      <c r="T20" t="n">
+        <v>225173</v>
+      </c>
+      <c r="U20" t="n">
+        <v>17185</v>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W20" t="b">
+        <v>1</v>
+      </c>
+      <c r="X20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB20" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12764,7 +13722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13899,6 +14857,163 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.636386</v>
+      </c>
+      <c r="T8" t="n">
+        <v>45357</v>
+      </c>
+      <c r="U8" t="n">
+        <v>15023</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13910,7 +15025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14529,6 +15644,94 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.70221</v>
+      </c>
+      <c r="E8" t="n">
+        <v>251976</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.70221</v>
+      </c>
+      <c r="G8" t="n">
+        <v>251976</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14540,7 +15743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14775,6 +15978,37 @@
         <v>4.926</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>43829</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.3063684</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.091</v>
+      </c>
+      <c r="F8" t="n">
+        <v>111277</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.63467</v>
+      </c>
+      <c r="H8" t="n">
+        <v>59</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -14787,7 +16021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15892,6 +17126,158 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.3063684</v>
+      </c>
+      <c r="T8" t="n">
+        <v>43829</v>
+      </c>
+      <c r="U8" t="n">
+        <v>12357</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15903,7 +17289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16516,6 +17902,93 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.63467</v>
+      </c>
+      <c r="E8" t="n">
+        <v>111277</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.63467</v>
+      </c>
+      <c r="G8" t="n">
+        <v>111277</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16527,7 +18000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16753,6 +18226,31 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.4816155</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>33710</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -16765,7 +18263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17822,6 +19320,150 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>350.57.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1787428673</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.4816155</v>
+      </c>
+      <c r="T8" t="n">
+        <v>46146</v>
+      </c>
+      <c r="U8" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17833,7 +19475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18398,6 +20040,85 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="E8" t="n">
+        <v>33710</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="G8" t="n">
+        <v>33710</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:32:27Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18409,7 +20130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19760,6 +21481,76 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4.73718</v>
+      </c>
+      <c r="E20" t="n">
+        <v>321539</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4.73718</v>
+      </c>
+      <c r="G20" t="n">
+        <v>321539</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19771,7 +21562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19997,6 +21788,34 @@
         <v>4.718</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>73829</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.6761904</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>57.094</v>
+      </c>
+      <c r="F8" t="n">
+        <v>113663</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.7176</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -20009,7 +21828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20970,6 +22789,134 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.6761904</v>
+      </c>
+      <c r="T8" t="n">
+        <v>73829</v>
+      </c>
+      <c r="U8" t="n">
+        <v>5912</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20981,7 +22928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21456,6 +23403,70 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.7176</v>
+      </c>
+      <c r="E8" t="n">
+        <v>113663</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.7176</v>
+      </c>
+      <c r="G8" t="n">
+        <v>113663</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21467,7 +23478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21702,6 +23713,37 @@
         <v>4.441</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>142922</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4.7577386</v>
+      </c>
+      <c r="D8" t="n">
+        <v>189</v>
+      </c>
+      <c r="E8" t="n">
+        <v>5.724</v>
+      </c>
+      <c r="F8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="H8" t="n">
+        <v>105</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4.541</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -21714,7 +23756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE7"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22927,167 +24969,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23133,66 +25036,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R8" t="n">
+        <v>4.7577386</v>
+      </c>
+      <c r="T8" t="n">
+        <v>142922</v>
+      </c>
+      <c r="U8" t="n">
+        <v>11058</v>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23239,65 +25346,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23344,65 +25451,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23449,65 +25556,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23554,65 +25661,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -23659,6 +25766,216 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-25
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$20</f>
+              <f>'ENBD Summary'!$A$2:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$20</f>
+              <f>'ENBD Summary'!$D$2:$D$21</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$20</f>
+              <f>'ENBD Summary'!$A$2:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$20</f>
+              <f>'ENBD Summary'!$H$2:$H$21</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$8</f>
+              <f>'ADCB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$8</f>
+              <f>'ADCB Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$8</f>
+              <f>'ADCB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$8</f>
+              <f>'ADCB Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$8</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$8</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$8</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$8</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$8</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$8</f>
+              <f>'ADIB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$8</f>
+              <f>'ADIB Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$8</f>
+              <f>'ADIB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$8</f>
+              <f>'ADIB Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$8</f>
+              <f>'ADIB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$8</f>
+              <f>'ADIB Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$8</f>
+              <f>'ADIB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$8</f>
+              <f>'ADIB Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$8</f>
+              <f>'FAB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$8</f>
+              <f>'FAB Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$8</f>
+              <f>'FAB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$8</f>
+              <f>'FAB Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$8</f>
+              <f>'FAB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$8</f>
+              <f>'FAB Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$8</f>
+              <f>'FAB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$8</f>
+              <f>'FAB Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$8</f>
+              <f>'RAK Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$8</f>
+              <f>'RAK Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$8</f>
+              <f>'RAK Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$8</f>
+              <f>'RAK Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$8</f>
+              <f>'RAK Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$8</f>
+              <f>'RAK Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$8</f>
+              <f>'RAK Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$8</f>
+              <f>'RAK Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$20</f>
+              <f>'ENBD Summary'!$A$2:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$20</f>
+              <f>'ENBD Summary'!$E$2:$E$21</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$20</f>
+              <f>'ENBD Summary'!$A$2:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$20</f>
+              <f>'ENBD Summary'!$I$2:$I$21</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$8</f>
+              <f>'EI Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$8</f>
+              <f>'EI Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$8</f>
+              <f>'EI Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$8</f>
+              <f>'EI Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$8</f>
+              <f>'EI Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$8</f>
+              <f>'EI Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$8</f>
+              <f>'EI Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$8</f>
+              <f>'EI Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$8</f>
+              <f>'MASHREQ Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$8</f>
+              <f>'MASHREQ Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$8</f>
+              <f>'MASHREQ Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$8</f>
+              <f>'MASHREQ Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$8</f>
+              <f>'MASHREQ Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$8</f>
+              <f>'MASHREQ Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$8</f>
+              <f>'MASHREQ Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$8</f>
+              <f>'MASHREQ Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$8</f>
+              <f>'WIO Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$8</f>
+              <f>'WIO Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$8</f>
+              <f>'WIO Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$8</f>
+              <f>'WIO Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$8</f>
+              <f>'WIO Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$8</f>
+              <f>'WIO Summary'!$E$2:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$8</f>
+              <f>'WIO Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$8</f>
+              <f>'WIO Summary'!$I$2:$I$9</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$8</f>
+              <f>'ADCB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$8</f>
+              <f>'ADCB Summary'!$D$2:$D$9</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$8</f>
+              <f>'ADCB Summary'!$A$2:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$8</f>
+              <f>'ADCB Summary'!$H$2:$H$9</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4232,6 +4232,37 @@
         <v>3.531</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>225179</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4.693302</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" t="n">
+        <v>-18.289</v>
+      </c>
+      <c r="F21" t="n">
+        <v>321554</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4.7371</v>
+      </c>
+      <c r="H21" t="n">
+        <v>15</v>
+      </c>
+      <c r="I21" t="n">
+        <v>3.022</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4244,7 +4275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4510,6 +4541,37 @@
         <v>4.989</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5788</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.6084657</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6.398</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6684</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.80729</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3.003</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4522,7 +4584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5716,6 +5778,149 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.6084657</v>
+      </c>
+      <c r="T9" t="n">
+        <v>5788</v>
+      </c>
+      <c r="U9" t="n">
+        <v>524</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5727,7 +5932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6364,6 +6569,84 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.80729</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6684</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80729</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6684</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6375,7 +6658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6611,6 +6894,31 @@
         <v>5.247</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>64315</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.2174926</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>113007</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6623,7 +6931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7817,6 +8125,149 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.2174926</v>
+      </c>
+      <c r="T9" t="n">
+        <v>64315</v>
+      </c>
+      <c r="U9" t="n">
+        <v>15247</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7828,7 +8279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8472,6 +8923,85 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="E9" t="n">
+        <v>113007</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="G9" t="n">
+        <v>113007</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8483,7 +9013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8749,6 +9279,37 @@
         <v>4.636</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>73566</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.690013</v>
+      </c>
+      <c r="D9" t="n">
+        <v>119</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.696</v>
+      </c>
+      <c r="F9" t="n">
+        <v>74850</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.47279</v>
+      </c>
+      <c r="H9" t="n">
+        <v>146</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8761,7 +9322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9976,6 +10537,152 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.690013</v>
+      </c>
+      <c r="T9" t="n">
+        <v>73566</v>
+      </c>
+      <c r="U9" t="n">
+        <v>4854</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9987,7 +10694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10645,6 +11352,87 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.47279</v>
+      </c>
+      <c r="E9" t="n">
+        <v>74850</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.47279</v>
+      </c>
+      <c r="G9" t="n">
+        <v>74850</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10656,7 +11444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10922,6 +11710,37 @@
         <v>3.731</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>45365</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.636097</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.998</v>
+      </c>
+      <c r="F9" t="n">
+        <v>252037</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.70214</v>
+      </c>
+      <c r="H9" t="n">
+        <v>61</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.413</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10934,7 +11753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE20"/>
+  <dimension ref="A1:AE21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13711,6 +14530,142 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R21" t="n">
+        <v>4.693302</v>
+      </c>
+      <c r="T21" t="n">
+        <v>225179</v>
+      </c>
+      <c r="U21" t="n">
+        <v>17191</v>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W21" t="b">
+        <v>1</v>
+      </c>
+      <c r="X21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13722,7 +14677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15014,6 +15969,163 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.636097</v>
+      </c>
+      <c r="T9" t="n">
+        <v>45365</v>
+      </c>
+      <c r="U9" t="n">
+        <v>15029</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15025,7 +16137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15732,6 +16844,94 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.70214</v>
+      </c>
+      <c r="E9" t="n">
+        <v>252037</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.70214</v>
+      </c>
+      <c r="G9" t="n">
+        <v>252037</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15743,7 +16943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16009,6 +17209,37 @@
         <v>4.333</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>43835</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.306851</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7.832</v>
+      </c>
+      <c r="F9" t="n">
+        <v>111313</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.63455</v>
+      </c>
+      <c r="H9" t="n">
+        <v>36</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.264</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -16021,7 +17252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17278,6 +18509,158 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.306851</v>
+      </c>
+      <c r="T9" t="n">
+        <v>43835</v>
+      </c>
+      <c r="U9" t="n">
+        <v>12360</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17289,7 +18672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17989,6 +19372,93 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.63455</v>
+      </c>
+      <c r="E9" t="n">
+        <v>111313</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.63455</v>
+      </c>
+      <c r="G9" t="n">
+        <v>111313</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18000,7 +19470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18251,6 +19721,37 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>46149</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.4813476</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.361</v>
+      </c>
+      <c r="F9" t="n">
+        <v>33711</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.635</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -18263,7 +19764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19464,6 +20965,150 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>350.57.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1787428673</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.4813476</v>
+      </c>
+      <c r="T9" t="n">
+        <v>46149</v>
+      </c>
+      <c r="U9" t="n">
+        <v>3262</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19475,7 +21120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20119,6 +21764,85 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="E9" t="n">
+        <v>33711</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.63518</v>
+      </c>
+      <c r="G9" t="n">
+        <v>33711</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:32:27Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20130,7 +21854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21551,6 +23275,76 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>4.7371</v>
+      </c>
+      <c r="E21" t="n">
+        <v>321554</v>
+      </c>
+      <c r="F21" t="n">
+        <v>4.7371</v>
+      </c>
+      <c r="G21" t="n">
+        <v>321554</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21562,7 +23356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21816,6 +23610,37 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>73830</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.675534</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-43.786</v>
+      </c>
+      <c r="F9" t="n">
+        <v>113664</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6.991</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -21828,7 +23653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22917,6 +24742,134 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.675534</v>
+      </c>
+      <c r="T9" t="n">
+        <v>73830</v>
+      </c>
+      <c r="U9" t="n">
+        <v>5913</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22928,7 +24881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23467,6 +25420,70 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="E9" t="n">
+        <v>113664</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.71762</v>
+      </c>
+      <c r="G9" t="n">
+        <v>113664</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23478,7 +25495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23744,6 +25761,37 @@
         <v>4.541</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>143089</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4.756282</v>
+      </c>
+      <c r="D9" t="n">
+        <v>167</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="F9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="H9" t="n">
+        <v>73</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4.671</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -23756,7 +25804,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25139,167 +27187,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25345,66 +27254,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4.756282</v>
+      </c>
+      <c r="T9" t="n">
+        <v>143089</v>
+      </c>
+      <c r="U9" t="n">
+        <v>11066</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25451,65 +27564,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25556,65 +27669,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25661,65 +27774,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25766,65 +27879,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25871,65 +27984,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -25976,6 +28089,216 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-26
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$21</f>
+              <f>'ENBD Summary'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$21</f>
+              <f>'ENBD Summary'!$D$2:$D$22</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$21</f>
+              <f>'ENBD Summary'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$21</f>
+              <f>'ENBD Summary'!$H$2:$H$22</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$9</f>
+              <f>'ADCB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$9</f>
+              <f>'ADCB Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$9</f>
+              <f>'ADCB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$9</f>
+              <f>'ADCB Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$9</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$9</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$9</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$9</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$9</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$9</f>
+              <f>'ADIB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$9</f>
+              <f>'ADIB Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$9</f>
+              <f>'ADIB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$9</f>
+              <f>'ADIB Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$9</f>
+              <f>'ADIB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$9</f>
+              <f>'ADIB Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$9</f>
+              <f>'ADIB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$9</f>
+              <f>'ADIB Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$9</f>
+              <f>'FAB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$9</f>
+              <f>'FAB Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$9</f>
+              <f>'FAB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$9</f>
+              <f>'FAB Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$9</f>
+              <f>'FAB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$9</f>
+              <f>'FAB Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$9</f>
+              <f>'FAB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$9</f>
+              <f>'FAB Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$9</f>
+              <f>'RAK Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$9</f>
+              <f>'RAK Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$9</f>
+              <f>'RAK Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$9</f>
+              <f>'RAK Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$9</f>
+              <f>'RAK Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$9</f>
+              <f>'RAK Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$9</f>
+              <f>'RAK Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$9</f>
+              <f>'RAK Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$21</f>
+              <f>'ENBD Summary'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$21</f>
+              <f>'ENBD Summary'!$E$2:$E$22</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$21</f>
+              <f>'ENBD Summary'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$21</f>
+              <f>'ENBD Summary'!$I$2:$I$22</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$9</f>
+              <f>'EI Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$9</f>
+              <f>'EI Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$9</f>
+              <f>'EI Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$9</f>
+              <f>'EI Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$9</f>
+              <f>'EI Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$9</f>
+              <f>'EI Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$9</f>
+              <f>'EI Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$9</f>
+              <f>'EI Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$9</f>
+              <f>'MASHREQ Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$9</f>
+              <f>'MASHREQ Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$9</f>
+              <f>'MASHREQ Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$9</f>
+              <f>'MASHREQ Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$9</f>
+              <f>'MASHREQ Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$9</f>
+              <f>'MASHREQ Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$9</f>
+              <f>'MASHREQ Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$9</f>
+              <f>'MASHREQ Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$9</f>
+              <f>'WIO Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$9</f>
+              <f>'WIO Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$9</f>
+              <f>'WIO Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$9</f>
+              <f>'WIO Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$9</f>
+              <f>'WIO Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$9</f>
+              <f>'WIO Summary'!$E$2:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$9</f>
+              <f>'WIO Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$9</f>
+              <f>'WIO Summary'!$I$2:$I$10</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$9</f>
+              <f>'ADCB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$9</f>
+              <f>'ADCB Summary'!$D$2:$D$10</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$9</f>
+              <f>'ADCB Summary'!$A$2:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$9</f>
+              <f>'ADCB Summary'!$H$2:$H$10</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4263,6 +4263,37 @@
         <v>3.022</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>225185</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4.692825</v>
+      </c>
+      <c r="D22" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" t="n">
+        <v>-13.209</v>
+      </c>
+      <c r="F22" t="n">
+        <v>321563</v>
+      </c>
+      <c r="G22" t="n">
+        <v>4.73703</v>
+      </c>
+      <c r="H22" t="n">
+        <v>9</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2.236</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4275,7 +4306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4572,6 +4603,37 @@
         <v>3.003</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5795</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.593176</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-8.048999999999999</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6689</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.80759</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5.209</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4584,7 +4646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5921,6 +5983,149 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1786091427</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.593176</v>
+      </c>
+      <c r="T10" t="n">
+        <v>5795</v>
+      </c>
+      <c r="U10" t="n">
+        <v>525</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5932,7 +6137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6647,6 +6852,84 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.80759</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6689</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.80759</v>
+      </c>
+      <c r="G10" t="n">
+        <v>6689</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-12T10:10:32Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6658,7 +6941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6919,6 +7202,34 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>64313</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.2174926</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.682</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -6931,7 +7242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8268,6 +8579,149 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.2174926</v>
+      </c>
+      <c r="T10" t="n">
+        <v>64313</v>
+      </c>
+      <c r="U10" t="n">
+        <v>15247</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8279,7 +8733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9002,6 +9456,85 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="E10" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="G10" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9013,7 +9546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9310,6 +9843,37 @@
         <v>4.57</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>73761</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.6777797</v>
+      </c>
+      <c r="D10" t="n">
+        <v>195</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="F10" t="n">
+        <v>75041</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.47315</v>
+      </c>
+      <c r="H10" t="n">
+        <v>191</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.614</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9322,7 +9886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10683,6 +11247,152 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1787127823</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.6777797</v>
+      </c>
+      <c r="T10" t="n">
+        <v>73761</v>
+      </c>
+      <c r="U10" t="n">
+        <v>4873</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10694,7 +11404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11433,6 +12143,87 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.47315</v>
+      </c>
+      <c r="E10" t="n">
+        <v>75041</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.47315</v>
+      </c>
+      <c r="G10" t="n">
+        <v>75041</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11444,7 +12235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11741,6 +12532,37 @@
         <v>4.413</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.6362967</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="F10" t="n">
+        <v>252090</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.70202</v>
+      </c>
+      <c r="H10" t="n">
+        <v>53</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.131</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11753,7 +12575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE21"/>
+  <dimension ref="A1:AE22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14666,6 +15488,142 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>1786695286</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R22" t="n">
+        <v>4.692825</v>
+      </c>
+      <c r="T22" t="n">
+        <v>225185</v>
+      </c>
+      <c r="U22" t="n">
+        <v>17197</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W22" t="b">
+        <v>1</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14677,7 +15635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16126,6 +17084,163 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.6362967</v>
+      </c>
+      <c r="T10" t="n">
+        <v>45372</v>
+      </c>
+      <c r="U10" t="n">
+        <v>15035</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16137,7 +17252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16932,6 +18047,94 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.70202</v>
+      </c>
+      <c r="E10" t="n">
+        <v>252090</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.70202</v>
+      </c>
+      <c r="G10" t="n">
+        <v>252090</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16943,7 +18146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17240,6 +18443,37 @@
         <v>4.264</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>43844</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.3088403</v>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>13.998</v>
+      </c>
+      <c r="F10" t="n">
+        <v>111379</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.63447</v>
+      </c>
+      <c r="H10" t="n">
+        <v>66</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -17252,7 +18486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18661,6 +19895,158 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.3088403</v>
+      </c>
+      <c r="T10" t="n">
+        <v>43844</v>
+      </c>
+      <c r="U10" t="n">
+        <v>12367</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18672,7 +20058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19459,6 +20845,93 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.63447</v>
+      </c>
+      <c r="E10" t="n">
+        <v>111379</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.63447</v>
+      </c>
+      <c r="G10" t="n">
+        <v>111379</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19470,7 +20943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19752,6 +21225,31 @@
         <v>4.635</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>46149</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.4799557</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>33709</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -19764,7 +21262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21109,6 +22607,150 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>350.57.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1787428673</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.4799557</v>
+      </c>
+      <c r="T10" t="n">
+        <v>46149</v>
+      </c>
+      <c r="U10" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21120,7 +22762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21843,6 +23485,85 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="E10" t="n">
+        <v>33709</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="G10" t="n">
+        <v>33709</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:32:27Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21854,7 +23575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23345,6 +25066,76 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>4.73703</v>
+      </c>
+      <c r="E22" t="n">
+        <v>321563</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4.73703</v>
+      </c>
+      <c r="G22" t="n">
+        <v>321563</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23356,7 +25147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23641,6 +25432,34 @@
         <v>6.991</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>73826</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.675267</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F10" t="n">
+        <v>113669</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.71749</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1.762</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -23653,7 +25472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24870,6 +26689,134 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1786701688</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.675267</v>
+      </c>
+      <c r="T10" t="n">
+        <v>73826</v>
+      </c>
+      <c r="U10" t="n">
+        <v>5915</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24881,7 +26828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25484,6 +27431,70 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.71749</v>
+      </c>
+      <c r="E10" t="n">
+        <v>113669</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.71749</v>
+      </c>
+      <c r="G10" t="n">
+        <v>113669</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25495,7 +27506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25792,6 +27803,37 @@
         <v>4.671</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>143282</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.759106</v>
+      </c>
+      <c r="D10" t="n">
+        <v>193</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6.853</v>
+      </c>
+      <c r="F10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="H10" t="n">
+        <v>123</v>
+      </c>
+      <c r="I10" t="n">
+        <v>4.68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -25804,7 +27846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
+  <dimension ref="A1:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27357,167 +29399,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -27563,66 +29466,270 @@
 Dubai, UAE</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4.759106</v>
+      </c>
+      <c r="T10" t="n">
+        <v>143282</v>
+      </c>
+      <c r="U10" t="n">
+        <v>11077</v>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -27669,65 +29776,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -27774,65 +29881,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -27879,65 +29986,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -27984,65 +30091,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -28089,65 +30196,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -28194,65 +30301,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -28299,6 +30406,216 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-27
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$22</f>
+              <f>'ENBD Summary'!$A$2:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$22</f>
+              <f>'ENBD Summary'!$D$2:$D$23</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$22</f>
+              <f>'ENBD Summary'!$A$2:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$22</f>
+              <f>'ENBD Summary'!$H$2:$H$23</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$10</f>
+              <f>'ADCB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$10</f>
+              <f>'ADCB Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$10</f>
+              <f>'ADCB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$10</f>
+              <f>'ADCB Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$10</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$10</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$10</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$10</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$10</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$10</f>
+              <f>'ADIB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$10</f>
+              <f>'ADIB Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$10</f>
+              <f>'ADIB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$10</f>
+              <f>'ADIB Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$10</f>
+              <f>'ADIB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$10</f>
+              <f>'ADIB Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$10</f>
+              <f>'ADIB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$10</f>
+              <f>'ADIB Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$10</f>
+              <f>'FAB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$10</f>
+              <f>'FAB Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$10</f>
+              <f>'FAB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$10</f>
+              <f>'FAB Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$10</f>
+              <f>'FAB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$10</f>
+              <f>'FAB Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$10</f>
+              <f>'FAB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$10</f>
+              <f>'FAB Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$10</f>
+              <f>'RAK Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$10</f>
+              <f>'RAK Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$10</f>
+              <f>'RAK Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$10</f>
+              <f>'RAK Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$10</f>
+              <f>'RAK Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$10</f>
+              <f>'RAK Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$10</f>
+              <f>'RAK Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$10</f>
+              <f>'RAK Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$22</f>
+              <f>'ENBD Summary'!$A$2:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$22</f>
+              <f>'ENBD Summary'!$E$2:$E$23</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$22</f>
+              <f>'ENBD Summary'!$A$2:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$22</f>
+              <f>'ENBD Summary'!$I$2:$I$23</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$10</f>
+              <f>'EI Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$10</f>
+              <f>'EI Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$10</f>
+              <f>'EI Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$10</f>
+              <f>'EI Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$10</f>
+              <f>'EI Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$10</f>
+              <f>'EI Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$10</f>
+              <f>'EI Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$10</f>
+              <f>'EI Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$10</f>
+              <f>'MASHREQ Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$10</f>
+              <f>'MASHREQ Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$10</f>
+              <f>'MASHREQ Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$10</f>
+              <f>'MASHREQ Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$10</f>
+              <f>'MASHREQ Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$10</f>
+              <f>'MASHREQ Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$10</f>
+              <f>'MASHREQ Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$10</f>
+              <f>'MASHREQ Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$10</f>
+              <f>'WIO Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$10</f>
+              <f>'WIO Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$10</f>
+              <f>'WIO Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$10</f>
+              <f>'WIO Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$10</f>
+              <f>'WIO Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$10</f>
+              <f>'WIO Summary'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$10</f>
+              <f>'WIO Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$10</f>
+              <f>'WIO Summary'!$I$2:$I$11</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$10</f>
+              <f>'ADCB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$10</f>
+              <f>'ADCB Summary'!$D$2:$D$11</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$10</f>
+              <f>'ADCB Summary'!$A$2:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$10</f>
+              <f>'ADCB Summary'!$H$2:$H$11</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4294,6 +4294,37 @@
         <v>2.236</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>225191</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4.6926136</v>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="n">
+        <v>-3.241</v>
+      </c>
+      <c r="F23" t="n">
+        <v>321585</v>
+      </c>
+      <c r="G23" t="n">
+        <v>4.73693</v>
+      </c>
+      <c r="H23" t="n">
+        <v>22</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3.275</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4306,7 +4337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4634,6 +4665,37 @@
         <v>5.209</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5801</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.592208</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.657</v>
+      </c>
+      <c r="F11" t="n">
+        <v>6691</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.80765</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5.008</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4646,7 +4708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6126,6 +6188,149 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.592208</v>
+      </c>
+      <c r="T11" t="n">
+        <v>5801</v>
+      </c>
+      <c r="U11" t="n">
+        <v>525</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6137,7 +6342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6930,6 +7135,84 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.80765</v>
+      </c>
+      <c r="E11" t="n">
+        <v>6691</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.80765</v>
+      </c>
+      <c r="G11" t="n">
+        <v>6691</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6941,7 +7224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7230,6 +7513,31 @@
         <v>4.682</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>64312</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.2173266</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7242,7 +7550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8722,6 +9030,149 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.2173266</v>
+      </c>
+      <c r="T11" t="n">
+        <v>64312</v>
+      </c>
+      <c r="U11" t="n">
+        <v>15247</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8733,7 +9184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9535,6 +9986,85 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="E11" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.68154</v>
+      </c>
+      <c r="G11" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9546,7 +10076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9874,6 +10404,37 @@
         <v>4.614</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>73968</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.675514</v>
+      </c>
+      <c r="D11" t="n">
+        <v>207</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.868</v>
+      </c>
+      <c r="F11" t="n">
+        <v>75308</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.47363</v>
+      </c>
+      <c r="H11" t="n">
+        <v>267</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.609</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9886,7 +10447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11393,6 +11954,152 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787764969</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.675514</v>
+      </c>
+      <c r="T11" t="n">
+        <v>73968</v>
+      </c>
+      <c r="U11" t="n">
+        <v>4890</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11404,7 +12111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12224,6 +12931,87 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.47363</v>
+      </c>
+      <c r="E11" t="n">
+        <v>75308</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.47363</v>
+      </c>
+      <c r="G11" t="n">
+        <v>75308</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12235,7 +13023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12563,6 +13351,37 @@
         <v>4.131</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>45385</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.6362076</v>
+      </c>
+      <c r="D11" t="n">
+        <v>13</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.325</v>
+      </c>
+      <c r="F11" t="n">
+        <v>252168</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.70186</v>
+      </c>
+      <c r="H11" t="n">
+        <v>78</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.185</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -12575,7 +13394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE22"/>
+  <dimension ref="A1:AE23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15624,6 +16443,142 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R23" t="n">
+        <v>4.6926136</v>
+      </c>
+      <c r="T23" t="n">
+        <v>225191</v>
+      </c>
+      <c r="U23" t="n">
+        <v>17200</v>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W23" t="b">
+        <v>1</v>
+      </c>
+      <c r="X23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15635,7 +16590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17241,6 +18196,163 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.6362076</v>
+      </c>
+      <c r="T11" t="n">
+        <v>45385</v>
+      </c>
+      <c r="U11" t="n">
+        <v>15042</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17252,7 +18364,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18135,6 +19247,94 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.70186</v>
+      </c>
+      <c r="E11" t="n">
+        <v>252168</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.70186</v>
+      </c>
+      <c r="G11" t="n">
+        <v>252168</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18146,7 +19346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18474,6 +19674,37 @@
         <v>4.5</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>43854</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.304885</v>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-13.037</v>
+      </c>
+      <c r="F11" t="n">
+        <v>111460</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.6345</v>
+      </c>
+      <c r="H11" t="n">
+        <v>81</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.676</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -18486,7 +19717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20047,6 +21278,158 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.304885</v>
+      </c>
+      <c r="T11" t="n">
+        <v>43854</v>
+      </c>
+      <c r="U11" t="n">
+        <v>12371</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20058,7 +21441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20932,6 +22315,93 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.6345</v>
+      </c>
+      <c r="E11" t="n">
+        <v>111460</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.6345</v>
+      </c>
+      <c r="G11" t="n">
+        <v>111460</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20943,7 +22413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21250,6 +22720,31 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.4798107</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>33708</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -21262,7 +22757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22751,6 +24246,150 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.4798107</v>
+      </c>
+      <c r="T11" t="n">
+        <v>46148</v>
+      </c>
+      <c r="U11" t="n">
+        <v>3262</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22762,7 +24401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23564,6 +25203,85 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="E11" t="n">
+        <v>33708</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="G11" t="n">
+        <v>33708</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:32:27Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23575,7 +25293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25136,6 +26854,76 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>4.73693</v>
+      </c>
+      <c r="E23" t="n">
+        <v>321585</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4.73693</v>
+      </c>
+      <c r="G23" t="n">
+        <v>321585</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-08-17T10:38:47Z</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25147,7 +26935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25460,6 +27248,34 @@
         <v>1.762</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>73826</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.673349</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>113670</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.71742</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-3.239</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -25472,7 +27288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26817,6 +28633,134 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.673349</v>
+      </c>
+      <c r="T11" t="n">
+        <v>73826</v>
+      </c>
+      <c r="U11" t="n">
+        <v>5916</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26828,7 +28772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27495,6 +29439,70 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.71742</v>
+      </c>
+      <c r="E11" t="n">
+        <v>113670</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.71742</v>
+      </c>
+      <c r="G11" t="n">
+        <v>113670</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>26.8.2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-17T09:36:05Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27506,7 +29514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27834,6 +29842,37 @@
         <v>4.68</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>143478</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.757995</v>
+      </c>
+      <c r="D11" t="n">
+        <v>196</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.946</v>
+      </c>
+      <c r="F11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="H11" t="n">
+        <v>103</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4.669</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -27846,7 +29885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29569,167 +31608,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -29775,66 +31675,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R11" t="n">
+        <v>4.757995</v>
+      </c>
+      <c r="T11" t="n">
+        <v>143478</v>
+      </c>
+      <c r="U11" t="n">
+        <v>11090</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -29881,65 +31985,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -29986,65 +32090,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30091,65 +32195,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30196,65 +32300,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30301,65 +32405,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30406,65 +32510,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30511,65 +32615,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -30616,6 +32720,216 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-28
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$23</f>
+              <f>'ENBD Summary'!$A$2:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$23</f>
+              <f>'ENBD Summary'!$D$2:$D$24</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$23</f>
+              <f>'ENBD Summary'!$A$2:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$23</f>
+              <f>'ENBD Summary'!$H$2:$H$24</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$11</f>
+              <f>'ADCB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$11</f>
+              <f>'ADCB Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$11</f>
+              <f>'ADCB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$11</f>
+              <f>'ADCB Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$11</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$11</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$11</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$11</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$11</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$11</f>
+              <f>'ADIB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$11</f>
+              <f>'ADIB Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$11</f>
+              <f>'ADIB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$11</f>
+              <f>'ADIB Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$11</f>
+              <f>'ADIB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$11</f>
+              <f>'ADIB Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$11</f>
+              <f>'ADIB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$11</f>
+              <f>'ADIB Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$11</f>
+              <f>'FAB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$11</f>
+              <f>'FAB Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$11</f>
+              <f>'FAB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$11</f>
+              <f>'FAB Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$11</f>
+              <f>'FAB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$11</f>
+              <f>'FAB Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$11</f>
+              <f>'FAB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$11</f>
+              <f>'FAB Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$11</f>
+              <f>'RAK Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$11</f>
+              <f>'RAK Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$11</f>
+              <f>'RAK Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$11</f>
+              <f>'RAK Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$11</f>
+              <f>'RAK Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$11</f>
+              <f>'RAK Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$11</f>
+              <f>'RAK Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$11</f>
+              <f>'RAK Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$23</f>
+              <f>'ENBD Summary'!$A$2:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$23</f>
+              <f>'ENBD Summary'!$E$2:$E$24</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$23</f>
+              <f>'ENBD Summary'!$A$2:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$23</f>
+              <f>'ENBD Summary'!$I$2:$I$24</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$11</f>
+              <f>'EI Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$11</f>
+              <f>'EI Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$11</f>
+              <f>'EI Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$11</f>
+              <f>'EI Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$11</f>
+              <f>'EI Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$11</f>
+              <f>'EI Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$11</f>
+              <f>'EI Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$11</f>
+              <f>'EI Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$11</f>
+              <f>'MASHREQ Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$11</f>
+              <f>'MASHREQ Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$11</f>
+              <f>'MASHREQ Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$11</f>
+              <f>'MASHREQ Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$11</f>
+              <f>'MASHREQ Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$11</f>
+              <f>'MASHREQ Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$11</f>
+              <f>'MASHREQ Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$11</f>
+              <f>'MASHREQ Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$11</f>
+              <f>'WIO Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$11</f>
+              <f>'WIO Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$11</f>
+              <f>'WIO Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$11</f>
+              <f>'WIO Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$11</f>
+              <f>'WIO Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$11</f>
+              <f>'WIO Summary'!$E$2:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$11</f>
+              <f>'WIO Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$11</f>
+              <f>'WIO Summary'!$I$2:$I$12</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$11</f>
+              <f>'ADCB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$11</f>
+              <f>'ADCB Summary'!$D$2:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$11</f>
+              <f>'ADCB Summary'!$A$2:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$11</f>
+              <f>'ADCB Summary'!$H$2:$H$12</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4325,6 +4325,37 @@
         <v>3.275</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>225201</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4.6916966</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E24" t="n">
+        <v>-15.958</v>
+      </c>
+      <c r="F24" t="n">
+        <v>321591</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4.73686</v>
+      </c>
+      <c r="H24" t="n">
+        <v>6</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.985</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4337,7 +4368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4696,6 +4727,37 @@
         <v>5.008</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5806</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.586842</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-1.639</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6695</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.80822</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5.762</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4708,7 +4770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6331,6 +6393,149 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.586842</v>
+      </c>
+      <c r="T12" t="n">
+        <v>5806</v>
+      </c>
+      <c r="U12" t="n">
+        <v>525</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6342,7 +6547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7213,6 +7418,84 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.80822</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6695</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80822</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6695</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7224,7 +7507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7538,6 +7821,34 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>64310</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.217161</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>113009</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.68153</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3.551</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7550,7 +7861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9173,6 +9484,149 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.217161</v>
+      </c>
+      <c r="T12" t="n">
+        <v>64310</v>
+      </c>
+      <c r="U12" t="n">
+        <v>15247</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9184,7 +9638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10065,6 +10519,85 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.68153</v>
+      </c>
+      <c r="E12" t="n">
+        <v>113009</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.68153</v>
+      </c>
+      <c r="G12" t="n">
+        <v>113009</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10076,7 +10609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10435,6 +10968,37 @@
         <v>4.609</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>74206</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.6751113</v>
+      </c>
+      <c r="D12" t="n">
+        <v>238</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="F12" t="n">
+        <v>75600</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.47398</v>
+      </c>
+      <c r="H12" t="n">
+        <v>292</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.564</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -10447,7 +11011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12100,6 +12664,152 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787764969</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.6751113</v>
+      </c>
+      <c r="T12" t="n">
+        <v>74206</v>
+      </c>
+      <c r="U12" t="n">
+        <v>4908</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12111,7 +12821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13012,6 +13722,87 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.47398</v>
+      </c>
+      <c r="E12" t="n">
+        <v>75600</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.47398</v>
+      </c>
+      <c r="G12" t="n">
+        <v>75600</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13023,7 +13814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13382,6 +14173,37 @@
         <v>4.185</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>45403</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.6368756</v>
+      </c>
+      <c r="D12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6.321</v>
+      </c>
+      <c r="F12" t="n">
+        <v>252262</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.70174</v>
+      </c>
+      <c r="H12" t="n">
+        <v>94</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13394,7 +14216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE23"/>
+  <dimension ref="A1:AE24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16579,6 +17401,142 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R24" t="n">
+        <v>4.6916966</v>
+      </c>
+      <c r="T24" t="n">
+        <v>225201</v>
+      </c>
+      <c r="U24" t="n">
+        <v>17205</v>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W24" t="b">
+        <v>1</v>
+      </c>
+      <c r="X24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z24" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16590,7 +17548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18353,6 +19311,163 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.6368756</v>
+      </c>
+      <c r="T12" t="n">
+        <v>45403</v>
+      </c>
+      <c r="U12" t="n">
+        <v>15046</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18364,7 +19479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19335,6 +20450,94 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.70174</v>
+      </c>
+      <c r="E12" t="n">
+        <v>252262</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.70174</v>
+      </c>
+      <c r="G12" t="n">
+        <v>252262</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19346,7 +20549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19705,6 +20908,37 @@
         <v>4.676</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>43866</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.304784</v>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.936</v>
+      </c>
+      <c r="F12" t="n">
+        <v>111554</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="H12" t="n">
+        <v>94</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.718</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -19717,7 +20951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21430,6 +22664,158 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.304784</v>
+      </c>
+      <c r="T12" t="n">
+        <v>43866</v>
+      </c>
+      <c r="U12" t="n">
+        <v>12383</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21441,7 +22827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22402,6 +23788,93 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="E12" t="n">
+        <v>111554</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="G12" t="n">
+        <v>111554</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22413,7 +23886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22745,6 +24218,37 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.4792767</v>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-3.735</v>
+      </c>
+      <c r="F12" t="n">
+        <v>33710</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.63515</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.467</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -22757,7 +24261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24390,6 +25894,150 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.4792767</v>
+      </c>
+      <c r="T12" t="n">
+        <v>46151</v>
+      </c>
+      <c r="U12" t="n">
+        <v>3262</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24401,7 +26049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25282,6 +26930,85 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.63515</v>
+      </c>
+      <c r="E12" t="n">
+        <v>33710</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.63515</v>
+      </c>
+      <c r="G12" t="n">
+        <v>33710</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-27T14:25:32Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25293,7 +27020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26924,6 +28651,76 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>4.73686</v>
+      </c>
+      <c r="E24" t="n">
+        <v>321591</v>
+      </c>
+      <c r="F24" t="n">
+        <v>4.73686</v>
+      </c>
+      <c r="G24" t="n">
+        <v>321591</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:44:56Z</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26935,7 +28732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27276,6 +29073,37 @@
         <v>-3.239</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>73835</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.6738844</v>
+      </c>
+      <c r="D12" t="n">
+        <v>9</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9.066000000000001</v>
+      </c>
+      <c r="F12" t="n">
+        <v>113672</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3.012</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -27288,7 +29116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28761,6 +30589,134 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.6738844</v>
+      </c>
+      <c r="T12" t="n">
+        <v>73835</v>
+      </c>
+      <c r="U12" t="n">
+        <v>5918</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28772,7 +30728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29503,6 +31459,70 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="E12" t="n">
+        <v>113672</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="G12" t="n">
+        <v>113672</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:42:57Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -29514,7 +31534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29873,6 +31893,37 @@
         <v>4.669</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>143745</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4.7593575</v>
+      </c>
+      <c r="D12" t="n">
+        <v>267</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5.492</v>
+      </c>
+      <c r="F12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="H12" t="n">
+        <v>144</v>
+      </c>
+      <c r="I12" t="n">
+        <v>4.659</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -29885,7 +31936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31778,167 +33829,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -31984,66 +33896,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R12" t="n">
+        <v>4.7593575</v>
+      </c>
+      <c r="T12" t="n">
+        <v>143745</v>
+      </c>
+      <c r="U12" t="n">
+        <v>11102</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32090,65 +34206,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32195,65 +34311,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32300,65 +34416,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32405,65 +34521,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32510,65 +34626,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32615,65 +34731,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32720,65 +34836,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32825,65 +34941,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="E11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="G11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -32930,6 +35046,216 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="E12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-29
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$24</f>
+              <f>'ENBD Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$24</f>
+              <f>'ENBD Summary'!$D$2:$D$25</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$24</f>
+              <f>'ENBD Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$24</f>
+              <f>'ENBD Summary'!$H$2:$H$25</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$12</f>
+              <f>'ADCB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$12</f>
+              <f>'ADCB Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$12</f>
+              <f>'ADCB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$12</f>
+              <f>'ADCB Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$12</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$12</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$12</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$12</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$12</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$12</f>
+              <f>'ADIB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$12</f>
+              <f>'ADIB Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$12</f>
+              <f>'ADIB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$12</f>
+              <f>'ADIB Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$12</f>
+              <f>'ADIB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$12</f>
+              <f>'ADIB Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$12</f>
+              <f>'ADIB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$12</f>
+              <f>'ADIB Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$12</f>
+              <f>'FAB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$12</f>
+              <f>'FAB Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$12</f>
+              <f>'FAB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$12</f>
+              <f>'FAB Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$12</f>
+              <f>'FAB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$12</f>
+              <f>'FAB Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$12</f>
+              <f>'FAB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$12</f>
+              <f>'FAB Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$12</f>
+              <f>'RAK Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$12</f>
+              <f>'RAK Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$12</f>
+              <f>'RAK Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$12</f>
+              <f>'RAK Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$12</f>
+              <f>'RAK Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$12</f>
+              <f>'RAK Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$12</f>
+              <f>'RAK Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$12</f>
+              <f>'RAK Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$24</f>
+              <f>'ENBD Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$24</f>
+              <f>'ENBD Summary'!$E$2:$E$25</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$24</f>
+              <f>'ENBD Summary'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$24</f>
+              <f>'ENBD Summary'!$I$2:$I$25</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$12</f>
+              <f>'EI Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$12</f>
+              <f>'EI Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$12</f>
+              <f>'EI Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$12</f>
+              <f>'EI Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$12</f>
+              <f>'EI Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$12</f>
+              <f>'EI Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$12</f>
+              <f>'EI Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$12</f>
+              <f>'EI Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$12</f>
+              <f>'MASHREQ Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$12</f>
+              <f>'MASHREQ Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$12</f>
+              <f>'MASHREQ Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$12</f>
+              <f>'MASHREQ Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$12</f>
+              <f>'MASHREQ Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$12</f>
+              <f>'MASHREQ Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$12</f>
+              <f>'MASHREQ Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$12</f>
+              <f>'MASHREQ Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$12</f>
+              <f>'WIO Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$12</f>
+              <f>'WIO Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$12</f>
+              <f>'WIO Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$12</f>
+              <f>'WIO Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$12</f>
+              <f>'WIO Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$12</f>
+              <f>'WIO Summary'!$E$2:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$12</f>
+              <f>'WIO Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$12</f>
+              <f>'WIO Summary'!$I$2:$I$13</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$12</f>
+              <f>'ADCB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$12</f>
+              <f>'ADCB Summary'!$D$2:$D$13</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$12</f>
+              <f>'ADCB Summary'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$12</f>
+              <f>'ADCB Summary'!$H$2:$H$13</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4356,6 +4356,37 @@
         <v>0.985</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>225214</v>
+      </c>
+      <c r="C25" t="n">
+        <v>4.6908665</v>
+      </c>
+      <c r="D25" t="n">
+        <v>13</v>
+      </c>
+      <c r="E25" t="n">
+        <v>-9.689</v>
+      </c>
+      <c r="F25" t="n">
+        <v>321606</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4.73681</v>
+      </c>
+      <c r="H25" t="n">
+        <v>15</v>
+      </c>
+      <c r="I25" t="n">
+        <v>3.665</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4368,7 +4399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4758,6 +4789,37 @@
         <v>5.762</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5814</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.5894737</v>
+      </c>
+      <c r="D13" t="n">
+        <v>8</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6.499</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6705</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.80761</v>
+      </c>
+      <c r="H13" t="n">
+        <v>10</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.399</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4770,7 +4832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6536,6 +6598,149 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.5894737</v>
+      </c>
+      <c r="T13" t="n">
+        <v>5814</v>
+      </c>
+      <c r="U13" t="n">
+        <v>526</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6547,7 +6752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7496,6 +7701,84 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.80761</v>
+      </c>
+      <c r="E13" t="n">
+        <v>6705</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.80761</v>
+      </c>
+      <c r="G13" t="n">
+        <v>6705</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7507,7 +7790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7849,6 +8132,37 @@
         <v>3.551</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>64311</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.2166457</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-28.922</v>
+      </c>
+      <c r="F13" t="n">
+        <v>113011</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.68157</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>6.942</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -7861,7 +8175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9627,6 +9941,149 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.2166457</v>
+      </c>
+      <c r="T13" t="n">
+        <v>64311</v>
+      </c>
+      <c r="U13" t="n">
+        <v>15248</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9638,7 +10095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10598,6 +11055,85 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.68157</v>
+      </c>
+      <c r="E13" t="n">
+        <v>113011</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.68157</v>
+      </c>
+      <c r="G13" t="n">
+        <v>113011</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10609,7 +11145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10999,6 +11535,37 @@
         <v>4.564</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>74468</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.667751</v>
+      </c>
+      <c r="D13" t="n">
+        <v>262</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.583</v>
+      </c>
+      <c r="F13" t="n">
+        <v>75971</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.47502</v>
+      </c>
+      <c r="H13" t="n">
+        <v>371</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.687</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11011,7 +11578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12810,6 +13377,152 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787764969</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.667751</v>
+      </c>
+      <c r="T13" t="n">
+        <v>74468</v>
+      </c>
+      <c r="U13" t="n">
+        <v>4921</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12821,7 +13534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13803,6 +14516,87 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.47502</v>
+      </c>
+      <c r="E13" t="n">
+        <v>75971</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.47502</v>
+      </c>
+      <c r="G13" t="n">
+        <v>75971</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13814,7 +14608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14204,6 +14998,37 @@
         <v>4.38</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>45420</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.6347613</v>
+      </c>
+      <c r="D13" t="n">
+        <v>17</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-1.012</v>
+      </c>
+      <c r="F13" t="n">
+        <v>252434</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.70153</v>
+      </c>
+      <c r="H13" t="n">
+        <v>172</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.394</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -14216,7 +15041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE24"/>
+  <dimension ref="A1:AE25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17537,6 +18362,142 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R25" t="n">
+        <v>4.6908665</v>
+      </c>
+      <c r="T25" t="n">
+        <v>225214</v>
+      </c>
+      <c r="U25" t="n">
+        <v>17208</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W25" t="b">
+        <v>1</v>
+      </c>
+      <c r="X25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z25" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17548,7 +18509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19468,6 +20429,163 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.6347613</v>
+      </c>
+      <c r="T13" t="n">
+        <v>45420</v>
+      </c>
+      <c r="U13" t="n">
+        <v>15050</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -19479,7 +20597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20538,6 +21656,94 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.70153</v>
+      </c>
+      <c r="E13" t="n">
+        <v>252434</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.70153</v>
+      </c>
+      <c r="G13" t="n">
+        <v>252434</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20549,7 +21755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20939,6 +22145,37 @@
         <v>4.718</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>43889</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.3066134</v>
+      </c>
+      <c r="D13" t="n">
+        <v>23</v>
+      </c>
+      <c r="E13" t="n">
+        <v>7.796</v>
+      </c>
+      <c r="F13" t="n">
+        <v>111676</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.63474</v>
+      </c>
+      <c r="H13" t="n">
+        <v>122</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -20951,7 +22188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22816,6 +24053,158 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.3066134</v>
+      </c>
+      <c r="T13" t="n">
+        <v>43889</v>
+      </c>
+      <c r="U13" t="n">
+        <v>12392</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22827,7 +24216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23875,6 +25264,93 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.63474</v>
+      </c>
+      <c r="E13" t="n">
+        <v>111676</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.63474</v>
+      </c>
+      <c r="G13" t="n">
+        <v>111676</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23886,7 +25362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24249,6 +25725,31 @@
         <v>4.467</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.4794216</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>33708</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -24261,7 +25762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26038,6 +27539,150 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.4794216</v>
+      </c>
+      <c r="T13" t="n">
+        <v>46151</v>
+      </c>
+      <c r="U13" t="n">
+        <v>3262</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -26049,7 +27694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27009,6 +28654,85 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="E13" t="n">
+        <v>33708</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.63516</v>
+      </c>
+      <c r="G13" t="n">
+        <v>33708</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-27T14:25:32Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27020,7 +28744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28721,6 +30445,76 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>4.73681</v>
+      </c>
+      <c r="E25" t="n">
+        <v>321606</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.73681</v>
+      </c>
+      <c r="G25" t="n">
+        <v>321606</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:44:56Z</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28732,7 +30526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29104,6 +30898,37 @@
         <v>3.012</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>73839</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.672349</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-23.669</v>
+      </c>
+      <c r="F13" t="n">
+        <v>113674</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.71738</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.149</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -29116,7 +30941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30717,6 +32542,134 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.672349</v>
+      </c>
+      <c r="T13" t="n">
+        <v>73839</v>
+      </c>
+      <c r="U13" t="n">
+        <v>5918</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30728,7 +32681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31523,6 +33476,70 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.71738</v>
+      </c>
+      <c r="E13" t="n">
+        <v>113674</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.71738</v>
+      </c>
+      <c r="G13" t="n">
+        <v>113674</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:42:57Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -31534,7 +33551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31924,6 +33941,37 @@
         <v>4.659</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>143974</v>
+      </c>
+      <c r="C13" t="n">
+        <v>4.757745</v>
+      </c>
+      <c r="D13" t="n">
+        <v>229</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.746</v>
+      </c>
+      <c r="F13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="H13" t="n">
+        <v>136</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4.498</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -31936,7 +33984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33999,167 +36047,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34205,66 +36114,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R13" t="n">
+        <v>4.757745</v>
+      </c>
+      <c r="T13" t="n">
+        <v>143974</v>
+      </c>
+      <c r="U13" t="n">
+        <v>11114</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W13" t="b">
+        <v>1</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34311,65 +36424,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34416,65 +36529,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34521,65 +36634,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34626,65 +36739,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34731,65 +36844,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34836,65 +36949,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -34941,65 +37054,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -35046,65 +37159,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="E11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="G11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -35151,65 +37264,65 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="E12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="F12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="G12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -35256,6 +37369,216 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="E12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="E13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="G13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-08-30
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -209,12 +209,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$25</f>
+              <f>'ENBD Summary'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$25</f>
+              <f>'ENBD Summary'!$D$2:$D$26</f>
             </numRef>
           </val>
         </ser>
@@ -241,12 +241,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$25</f>
+              <f>'ENBD Summary'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$25</f>
+              <f>'ENBD Summary'!$H$2:$H$26</f>
             </numRef>
           </val>
         </ser>
@@ -360,12 +360,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$13</f>
+              <f>'ADCB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$13</f>
+              <f>'ADCB Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -392,12 +392,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$13</f>
+              <f>'ADCB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$13</f>
+              <f>'ADCB Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -511,12 +511,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$13</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -543,12 +543,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$13</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -662,12 +662,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$13</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -694,12 +694,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$13</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$13</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -813,12 +813,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$13</f>
+              <f>'ADIB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$13</f>
+              <f>'ADIB Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -845,12 +845,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$13</f>
+              <f>'ADIB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$13</f>
+              <f>'ADIB Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -964,12 +964,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$13</f>
+              <f>'ADIB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$13</f>
+              <f>'ADIB Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -996,12 +996,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$13</f>
+              <f>'ADIB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$13</f>
+              <f>'ADIB Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -1115,12 +1115,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$13</f>
+              <f>'FAB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$13</f>
+              <f>'FAB Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -1147,12 +1147,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$13</f>
+              <f>'FAB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$13</f>
+              <f>'FAB Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -1266,12 +1266,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$13</f>
+              <f>'FAB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$13</f>
+              <f>'FAB Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -1298,12 +1298,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$13</f>
+              <f>'FAB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$13</f>
+              <f>'FAB Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -1417,12 +1417,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$13</f>
+              <f>'RAK Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$13</f>
+              <f>'RAK Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -1449,12 +1449,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$13</f>
+              <f>'RAK Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$13</f>
+              <f>'RAK Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -1568,12 +1568,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$13</f>
+              <f>'RAK Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$13</f>
+              <f>'RAK Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -1600,12 +1600,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$13</f>
+              <f>'RAK Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$13</f>
+              <f>'RAK Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -1719,12 +1719,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$25</f>
+              <f>'ENBD Summary'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$25</f>
+              <f>'ENBD Summary'!$E$2:$E$26</f>
             </numRef>
           </val>
         </ser>
@@ -1751,12 +1751,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$25</f>
+              <f>'ENBD Summary'!$A$2:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$25</f>
+              <f>'ENBD Summary'!$I$2:$I$26</f>
             </numRef>
           </val>
         </ser>
@@ -1870,12 +1870,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$13</f>
+              <f>'EI Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$13</f>
+              <f>'EI Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -1902,12 +1902,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$13</f>
+              <f>'EI Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$13</f>
+              <f>'EI Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -2021,12 +2021,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$13</f>
+              <f>'EI Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$13</f>
+              <f>'EI Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -2053,12 +2053,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$13</f>
+              <f>'EI Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$13</f>
+              <f>'EI Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -2172,12 +2172,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$13</f>
+              <f>'MASHREQ Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$13</f>
+              <f>'MASHREQ Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -2204,12 +2204,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$13</f>
+              <f>'MASHREQ Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$13</f>
+              <f>'MASHREQ Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -2323,12 +2323,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$13</f>
+              <f>'MASHREQ Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$13</f>
+              <f>'MASHREQ Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -2355,12 +2355,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$13</f>
+              <f>'MASHREQ Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$13</f>
+              <f>'MASHREQ Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -2474,12 +2474,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$13</f>
+              <f>'WIO Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$13</f>
+              <f>'WIO Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -2506,12 +2506,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$13</f>
+              <f>'WIO Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$13</f>
+              <f>'WIO Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -2625,12 +2625,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$13</f>
+              <f>'WIO Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$13</f>
+              <f>'WIO Summary'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -2657,12 +2657,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$13</f>
+              <f>'WIO Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$13</f>
+              <f>'WIO Summary'!$I$2:$I$14</f>
             </numRef>
           </val>
         </ser>
@@ -2776,12 +2776,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$13</f>
+              <f>'ADCB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$13</f>
+              <f>'ADCB Summary'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -2808,12 +2808,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$13</f>
+              <f>'ADCB Summary'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$13</f>
+              <f>'ADCB Summary'!$H$2:$H$14</f>
             </numRef>
           </val>
         </ser>
@@ -3612,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4387,6 +4387,37 @@
         <v>3.665</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>225220</v>
+      </c>
+      <c r="C26" t="n">
+        <v>4.690778</v>
+      </c>
+      <c r="D26" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.369</v>
+      </c>
+      <c r="F26" t="n">
+        <v>321608</v>
+      </c>
+      <c r="G26" t="n">
+        <v>4.73678</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-0.08699999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4399,7 +4430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4820,6 +4851,37 @@
         <v>4.399</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.577428</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-12.931</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6714</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.80772</v>
+      </c>
+      <c r="H14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4832,7 +4894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6741,6 +6803,149 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1.70.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.577428</v>
+      </c>
+      <c r="T14" t="n">
+        <v>5818</v>
+      </c>
+      <c r="U14" t="n">
+        <v>527</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6752,7 +6957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7779,6 +7984,84 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.80772</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6714</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.80772</v>
+      </c>
+      <c r="G14" t="n">
+        <v>6714</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7790,7 +8073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8163,6 +8446,31 @@
         <v>6.942</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>64306</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.2159643</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8175,7 +8483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10084,6 +10392,149 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.2159643</v>
+      </c>
+      <c r="T14" t="n">
+        <v>64306</v>
+      </c>
+      <c r="U14" t="n">
+        <v>15246</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10095,7 +10546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11134,6 +11585,85 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="E14" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="G14" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11145,7 +11675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11566,6 +12096,37 @@
         <v>4.687</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>74657</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.666373</v>
+      </c>
+      <c r="D14" t="n">
+        <v>189</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.123</v>
+      </c>
+      <c r="F14" t="n">
+        <v>76186</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.47542</v>
+      </c>
+      <c r="H14" t="n">
+        <v>215</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.617</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -11578,7 +12139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13523,6 +14084,152 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787764969</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.666373</v>
+      </c>
+      <c r="T14" t="n">
+        <v>74657</v>
+      </c>
+      <c r="U14" t="n">
+        <v>4934</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -13534,7 +14241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14597,6 +15304,87 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.47542</v>
+      </c>
+      <c r="E14" t="n">
+        <v>76186</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.47542</v>
+      </c>
+      <c r="G14" t="n">
+        <v>76186</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-20T06:50:31Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14608,7 +15396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15029,6 +15817,37 @@
         <v>4.394</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>45432</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.635231</v>
+      </c>
+      <c r="D14" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6.413</v>
+      </c>
+      <c r="F14" t="n">
+        <v>252504</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.70157</v>
+      </c>
+      <c r="H14" t="n">
+        <v>70</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.846</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -15041,7 +15860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE25"/>
+  <dimension ref="A1:AE26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18498,6 +19317,142 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R26" t="n">
+        <v>4.690778</v>
+      </c>
+      <c r="T26" t="n">
+        <v>225220</v>
+      </c>
+      <c r="U26" t="n">
+        <v>17209</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W26" t="b">
+        <v>1</v>
+      </c>
+      <c r="X26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z26" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA26" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18509,7 +19464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20586,6 +21541,163 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.635231</v>
+      </c>
+      <c r="T14" t="n">
+        <v>45432</v>
+      </c>
+      <c r="U14" t="n">
+        <v>15052</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20597,7 +21709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21744,6 +22856,94 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.70157</v>
+      </c>
+      <c r="E14" t="n">
+        <v>252504</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.70157</v>
+      </c>
+      <c r="G14" t="n">
+        <v>252504</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21755,7 +22955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22176,6 +23376,37 @@
         <v>4.79</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>43908</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.308465</v>
+      </c>
+      <c r="D14" t="n">
+        <v>19</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8.586</v>
+      </c>
+      <c r="F14" t="n">
+        <v>111742</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="H14" t="n">
+        <v>66</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.347</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -22188,7 +23419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24205,6 +25436,158 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.308465</v>
+      </c>
+      <c r="T14" t="n">
+        <v>43908</v>
+      </c>
+      <c r="U14" t="n">
+        <v>12392</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24216,7 +25599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25351,6 +26734,93 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="E14" t="n">
+        <v>111742</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.63457</v>
+      </c>
+      <c r="G14" t="n">
+        <v>111742</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25362,7 +26832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25750,6 +27220,37 @@
         <v>-2</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>46158</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.4798994</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="F14" t="n">
+        <v>33712</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.6352</v>
+      </c>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.972</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -25762,7 +27263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27683,6 +29184,150 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.4798994</v>
+      </c>
+      <c r="T14" t="n">
+        <v>46158</v>
+      </c>
+      <c r="U14" t="n">
+        <v>3262</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27694,7 +29339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28733,6 +30378,85 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.6352</v>
+      </c>
+      <c r="E14" t="n">
+        <v>33712</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.6352</v>
+      </c>
+      <c r="G14" t="n">
+        <v>33712</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-27T14:25:32Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28744,7 +30468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30515,6 +32239,76 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>4.73678</v>
+      </c>
+      <c r="E26" t="n">
+        <v>321608</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.73678</v>
+      </c>
+      <c r="G26" t="n">
+        <v>321608</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:44:56Z</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -30526,7 +32320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30929,6 +32723,34 @@
         <v>4.149</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>73841</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.6724024</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6.644</v>
+      </c>
+      <c r="F14" t="n">
+        <v>113673</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -30941,7 +32763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32670,6 +34492,134 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.6724024</v>
+      </c>
+      <c r="T14" t="n">
+        <v>73841</v>
+      </c>
+      <c r="U14" t="n">
+        <v>5920</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32681,7 +34631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33540,6 +35490,70 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="E14" t="n">
+        <v>113673</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.71739</v>
+      </c>
+      <c r="G14" t="n">
+        <v>113673</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:42:57Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33551,7 +35565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -33972,6 +35986,37 @@
         <v>4.498</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>144191</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.7581906</v>
+      </c>
+      <c r="D14" t="n">
+        <v>217</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5.054</v>
+      </c>
+      <c r="F14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="H14" t="n">
+        <v>112</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4.913</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -33984,7 +36029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36217,167 +38262,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36423,66 +38329,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1786726583</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R14" t="n">
+        <v>4.7581906</v>
+      </c>
+      <c r="T14" t="n">
+        <v>144191</v>
+      </c>
+      <c r="U14" t="n">
+        <v>11125</v>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W14" t="b">
+        <v>1</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36529,65 +38639,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36634,65 +38744,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36739,65 +38849,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36844,65 +38954,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -36949,65 +39059,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37054,65 +39164,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37159,65 +39269,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37264,65 +39374,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="E11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="G11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37369,65 +39479,65 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="E12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="F12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="G12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37474,65 +39584,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="E13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="G13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="D12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="E12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -37579,6 +39689,216 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="E13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="G13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="E14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="G14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily ratings update: 2026-09-01
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -218,12 +218,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$27</f>
+              <f>'ENBD Summary'!$A$2:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$27</f>
+              <f>'ENBD Summary'!$D$2:$D$28</f>
             </numRef>
           </val>
         </ser>
@@ -250,12 +250,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$27</f>
+              <f>'ENBD Summary'!$A$2:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$27</f>
+              <f>'ENBD Summary'!$H$2:$H$28</f>
             </numRef>
           </val>
         </ser>
@@ -369,12 +369,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$15</f>
+              <f>'ADCB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$15</f>
+              <f>'ADCB Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -401,12 +401,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$15</f>
+              <f>'ADCB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$15</f>
+              <f>'ADCB Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -520,12 +520,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$15</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$15</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -552,12 +552,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$15</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$15</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -671,12 +671,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$15</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$15</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -703,12 +703,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$15</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$15</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -822,12 +822,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$15</f>
+              <f>'ADIB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$15</f>
+              <f>'ADIB Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -854,12 +854,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$15</f>
+              <f>'ADIB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$15</f>
+              <f>'ADIB Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -973,12 +973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$15</f>
+              <f>'ADIB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$15</f>
+              <f>'ADIB Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -1005,12 +1005,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$15</f>
+              <f>'ADIB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$15</f>
+              <f>'ADIB Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -1124,12 +1124,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$15</f>
+              <f>'FAB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$15</f>
+              <f>'FAB Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -1156,12 +1156,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$15</f>
+              <f>'FAB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$15</f>
+              <f>'FAB Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -1275,12 +1275,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$15</f>
+              <f>'FAB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$15</f>
+              <f>'FAB Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -1307,12 +1307,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$15</f>
+              <f>'FAB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$15</f>
+              <f>'FAB Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -1426,12 +1426,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$15</f>
+              <f>'RAK Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$15</f>
+              <f>'RAK Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -1458,12 +1458,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$15</f>
+              <f>'RAK Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$15</f>
+              <f>'RAK Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -1577,12 +1577,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$15</f>
+              <f>'RAK Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$15</f>
+              <f>'RAK Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -1609,12 +1609,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$15</f>
+              <f>'RAK Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$15</f>
+              <f>'RAK Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -1728,12 +1728,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$27</f>
+              <f>'ENBD Summary'!$A$2:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$27</f>
+              <f>'ENBD Summary'!$E$2:$E$28</f>
             </numRef>
           </val>
         </ser>
@@ -1760,12 +1760,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$27</f>
+              <f>'ENBD Summary'!$A$2:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$27</f>
+              <f>'ENBD Summary'!$I$2:$I$28</f>
             </numRef>
           </val>
         </ser>
@@ -1879,12 +1879,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$15</f>
+              <f>'EI Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$15</f>
+              <f>'EI Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -1911,12 +1911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$15</f>
+              <f>'EI Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$15</f>
+              <f>'EI Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -2030,12 +2030,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$15</f>
+              <f>'EI Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$15</f>
+              <f>'EI Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -2062,12 +2062,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$15</f>
+              <f>'EI Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$15</f>
+              <f>'EI Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -2181,12 +2181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$15</f>
+              <f>'MASHREQ Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$15</f>
+              <f>'MASHREQ Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -2213,12 +2213,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$15</f>
+              <f>'MASHREQ Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$15</f>
+              <f>'MASHREQ Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -2332,12 +2332,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$15</f>
+              <f>'MASHREQ Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$15</f>
+              <f>'MASHREQ Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -2364,12 +2364,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$15</f>
+              <f>'MASHREQ Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$15</f>
+              <f>'MASHREQ Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -2483,12 +2483,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$15</f>
+              <f>'WIO Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$15</f>
+              <f>'WIO Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -2515,12 +2515,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$15</f>
+              <f>'WIO Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$15</f>
+              <f>'WIO Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -2634,12 +2634,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$15</f>
+              <f>'WIO Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$15</f>
+              <f>'WIO Summary'!$E$2:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -2666,12 +2666,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$15</f>
+              <f>'WIO Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$15</f>
+              <f>'WIO Summary'!$I$2:$I$16</f>
             </numRef>
           </val>
         </ser>
@@ -2785,12 +2785,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$15</f>
+              <f>'ADCB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$15</f>
+              <f>'ADCB Summary'!$D$2:$D$16</f>
             </numRef>
           </val>
         </ser>
@@ -2817,12 +2817,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$15</f>
+              <f>'ADCB Summary'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$15</f>
+              <f>'ADCB Summary'!$H$2:$H$16</f>
             </numRef>
           </val>
         </ser>
@@ -3621,7 +3621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4458,6 +4458,37 @@
         <v>3.358</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>225227</v>
+      </c>
+      <c r="C28" t="n">
+        <v>4.6901016</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>-23.523</v>
+      </c>
+      <c r="F28" t="n">
+        <v>321625</v>
+      </c>
+      <c r="G28" t="n">
+        <v>4.7367</v>
+      </c>
+      <c r="H28" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" t="n">
+        <v>3.129</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4470,7 +4501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7043,167 +7074,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7249,66 +7141,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>9.18.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787843891</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.757832</v>
+      </c>
+      <c r="T16" t="n">
+        <v>144498</v>
+      </c>
+      <c r="U16" t="n">
+        <v>11145</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7355,65 +7451,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7460,65 +7556,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7565,65 +7661,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7670,65 +7766,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7775,65 +7871,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7880,65 +7976,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7985,65 +8081,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8090,65 +8186,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="E11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="G11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8195,65 +8291,65 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="E12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="F12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="G12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8300,65 +8396,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="E13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="G13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="D12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="E12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8405,65 +8501,65 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>4.80234</v>
-      </c>
-      <c r="E14" t="n">
-        <v>138127</v>
-      </c>
-      <c r="F14" t="n">
-        <v>4.80234</v>
-      </c>
-      <c r="G14" t="n">
-        <v>138127</v>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="D13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="E13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="G13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8510,65 +8606,65 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>4.8022</v>
-      </c>
-      <c r="E15" t="n">
-        <v>138217</v>
-      </c>
-      <c r="F15" t="n">
-        <v>4.8022</v>
-      </c>
-      <c r="G15" t="n">
-        <v>138217</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="D14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="E14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="G14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8615,6 +8711,216 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4.8022</v>
+      </c>
+      <c r="E15" t="n">
+        <v>138217</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.8022</v>
+      </c>
+      <c r="G15" t="n">
+        <v>138217</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.80218</v>
+      </c>
+      <c r="E16" t="n">
+        <v>138299</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.80218</v>
+      </c>
+      <c r="G16" t="n">
+        <v>138299</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>9.18.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-31T13:26:41Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8722,7 +9028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9205,6 +9511,37 @@
         <v>4.999</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5826</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.6015625</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>10.691</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6733</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.80781</v>
+      </c>
+      <c r="H16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.494</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9217,7 +9554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11412,6 +11749,149 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.6015625</v>
+      </c>
+      <c r="T16" t="n">
+        <v>5826</v>
+      </c>
+      <c r="U16" t="n">
+        <v>527</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11423,7 +11903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12587,6 +13067,84 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.80781</v>
+      </c>
+      <c r="E16" t="n">
+        <v>6733</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.80781</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6733</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
 Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
@@ -12713,7 +13271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13142,6 +13700,31 @@
         <v>5.812</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>64307</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.2136626</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13154,7 +13737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15349,6 +15932,149 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.2136626</v>
+      </c>
+      <c r="T16" t="n">
+        <v>64307</v>
+      </c>
+      <c r="U16" t="n">
+        <v>15245</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15360,7 +16086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16557,6 +17283,85 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="E16" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="G16" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16568,7 +17373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE27"/>
+  <dimension ref="A1:AE28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20297,6 +21102,142 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R28" t="n">
+        <v>4.6901016</v>
+      </c>
+      <c r="T28" t="n">
+        <v>225227</v>
+      </c>
+      <c r="U28" t="n">
+        <v>17217</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W28" t="b">
+        <v>1</v>
+      </c>
+      <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z28" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA28" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20398,7 +21339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20881,6 +21822,37 @@
         <v>4.559</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>75030</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.6730328</v>
+      </c>
+      <c r="D16" t="n">
+        <v>162</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="F16" t="n">
+        <v>76695</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.4764</v>
+      </c>
+      <c r="H16" t="n">
+        <v>234</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.699</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -20893,7 +21865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23130,6 +24102,152 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1788059707</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.6730328</v>
+      </c>
+      <c r="T16" t="n">
+        <v>75030</v>
+      </c>
+      <c r="U16" t="n">
+        <v>4955</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23141,7 +24259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24344,6 +25462,87 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.4764</v>
+      </c>
+      <c r="E16" t="n">
+        <v>76695</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.4764</v>
+      </c>
+      <c r="G16" t="n">
+        <v>76695</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-31T15:36:25Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
 The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
@@ -24473,7 +25672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24956,6 +26155,37 @@
         <v>4.196</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>45456</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.6377873</v>
+      </c>
+      <c r="D16" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" t="n">
+        <v>14.105</v>
+      </c>
+      <c r="F16" t="n">
+        <v>252632</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.70141</v>
+      </c>
+      <c r="H16" t="n">
+        <v>58</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.614</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -24968,7 +26198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27359,6 +28589,163 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.6377873</v>
+      </c>
+      <c r="T16" t="n">
+        <v>45456</v>
+      </c>
+      <c r="U16" t="n">
+        <v>15057</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27370,7 +28757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28664,6 +30051,94 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.70141</v>
+      </c>
+      <c r="E16" t="n">
+        <v>252632</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.70141</v>
+      </c>
+      <c r="G16" t="n">
+        <v>252632</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
 Features include: 
@@ -28800,7 +30275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29283,6 +30758,37 @@
         <v>4.801</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>43928</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.3106794</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" t="n">
+        <v>14.703</v>
+      </c>
+      <c r="F16" t="n">
+        <v>111868</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="H16" t="n">
+        <v>59</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.938</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -29295,7 +30801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31206,6 +32712,76 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>4.7367</v>
+      </c>
+      <c r="E28" t="n">
+        <v>321625</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.7367</v>
+      </c>
+      <c r="G28" t="n">
+        <v>321625</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:44:56Z</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -31217,7 +32793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33538,6 +35114,158 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.3106794</v>
+      </c>
+      <c r="T16" t="n">
+        <v>43928</v>
+      </c>
+      <c r="U16" t="n">
+        <v>12404</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33549,7 +35277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34830,6 +36558,93 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="E16" t="n">
+        <v>111868</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.63483</v>
+      </c>
+      <c r="G16" t="n">
+        <v>111868</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Let’s bring the bank to YOU! 
 The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
@@ -34965,7 +36780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35412,6 +37227,34 @@
         <v>4.298</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>46158</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.480045</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>33721</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.63509</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3.961</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -35424,7 +37267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37633,6 +39476,150 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.480045</v>
+      </c>
+      <c r="T16" t="n">
+        <v>46158</v>
+      </c>
+      <c r="U16" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37644,7 +39631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38821,6 +40808,85 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.63509</v>
+      </c>
+      <c r="E16" t="n">
+        <v>33721</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.63509</v>
+      </c>
+      <c r="G16" t="n">
+        <v>33721</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-27T14:25:32Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Our app brings you a simple yet secure way to manage, move and grow your money.
 YOUR MONEY ON YOUR TERMS
@@ -39044,7 +41110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39503,6 +41569,34 @@
         <v>2.444</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>73833</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.670274</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-8</v>
+      </c>
+      <c r="F16" t="n">
+        <v>113675</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.71737</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.717</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -39515,7 +41609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -41500,6 +43594,134 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R16" t="n">
+        <v>4.670274</v>
+      </c>
+      <c r="T16" t="n">
+        <v>73833</v>
+      </c>
+      <c r="U16" t="n">
+        <v>5920</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W16" t="b">
+        <v>1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -41511,7 +43733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -42493,6 +44715,70 @@
         </is>
       </c>
       <c r="N15" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.71737</v>
+      </c>
+      <c r="E16" t="n">
+        <v>113675</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.71737</v>
+      </c>
+      <c r="G16" t="n">
+        <v>113675</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:42:57Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
         <is>
           <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
         </is>
@@ -42605,7 +44891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43088,6 +45374,37 @@
         <v>4.587</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>144498</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.757832</v>
+      </c>
+      <c r="D16" t="n">
+        <v>129</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.653</v>
+      </c>
+      <c r="F16" t="n">
+        <v>138299</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.80218</v>
+      </c>
+      <c r="H16" t="n">
+        <v>82</v>
+      </c>
+      <c r="I16" t="n">
+        <v>4.768</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Daily ratings update: 2026-09-02
</commit_message>
<xml_diff>
--- a/app_ratings_history.xlsx
+++ b/app_ratings_history.xlsx
@@ -218,12 +218,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$28</f>
+              <f>'ENBD Summary'!$A$2:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$D$2:$D$28</f>
+              <f>'ENBD Summary'!$D$2:$D$29</f>
             </numRef>
           </val>
         </ser>
@@ -250,12 +250,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$28</f>
+              <f>'ENBD Summary'!$A$2:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$H$2:$H$28</f>
+              <f>'ENBD Summary'!$H$2:$H$29</f>
             </numRef>
           </val>
         </ser>
@@ -369,12 +369,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$16</f>
+              <f>'ADCB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$E$2:$E$16</f>
+              <f>'ADCB Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -401,12 +401,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$16</f>
+              <f>'ADCB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$I$2:$I$16</f>
+              <f>'ADCB Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -520,12 +520,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$D$2:$D$16</f>
+              <f>'ADCB NEW Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -552,12 +552,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$H$2:$H$16</f>
+              <f>'ADCB NEW Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -671,12 +671,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$E$2:$E$16</f>
+              <f>'ADCB NEW Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -703,12 +703,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB NEW Summary'!$A$2:$A$16</f>
+              <f>'ADCB NEW Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB NEW Summary'!$I$2:$I$16</f>
+              <f>'ADCB NEW Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -822,12 +822,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$16</f>
+              <f>'ADIB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$D$2:$D$16</f>
+              <f>'ADIB Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -854,12 +854,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$16</f>
+              <f>'ADIB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$H$2:$H$16</f>
+              <f>'ADIB Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -973,12 +973,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$16</f>
+              <f>'ADIB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$E$2:$E$16</f>
+              <f>'ADIB Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -1005,12 +1005,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADIB Summary'!$A$2:$A$16</f>
+              <f>'ADIB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADIB Summary'!$I$2:$I$16</f>
+              <f>'ADIB Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -1124,12 +1124,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$16</f>
+              <f>'FAB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$D$2:$D$16</f>
+              <f>'FAB Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -1156,12 +1156,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$16</f>
+              <f>'FAB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$H$2:$H$16</f>
+              <f>'FAB Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -1275,12 +1275,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$16</f>
+              <f>'FAB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$E$2:$E$16</f>
+              <f>'FAB Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -1307,12 +1307,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'FAB Summary'!$A$2:$A$16</f>
+              <f>'FAB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'FAB Summary'!$I$2:$I$16</f>
+              <f>'FAB Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -1426,12 +1426,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$16</f>
+              <f>'RAK Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$D$2:$D$16</f>
+              <f>'RAK Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -1458,12 +1458,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$16</f>
+              <f>'RAK Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$H$2:$H$16</f>
+              <f>'RAK Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -1577,12 +1577,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$16</f>
+              <f>'RAK Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$E$2:$E$16</f>
+              <f>'RAK Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -1609,12 +1609,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'RAK Summary'!$A$2:$A$16</f>
+              <f>'RAK Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RAK Summary'!$I$2:$I$16</f>
+              <f>'RAK Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -1728,12 +1728,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$28</f>
+              <f>'ENBD Summary'!$A$2:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$E$2:$E$28</f>
+              <f>'ENBD Summary'!$E$2:$E$29</f>
             </numRef>
           </val>
         </ser>
@@ -1760,12 +1760,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ENBD Summary'!$A$2:$A$28</f>
+              <f>'ENBD Summary'!$A$2:$A$29</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ENBD Summary'!$I$2:$I$28</f>
+              <f>'ENBD Summary'!$I$2:$I$29</f>
             </numRef>
           </val>
         </ser>
@@ -1879,12 +1879,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$16</f>
+              <f>'EI Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$D$2:$D$16</f>
+              <f>'EI Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -1911,12 +1911,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$16</f>
+              <f>'EI Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$H$2:$H$16</f>
+              <f>'EI Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -2030,12 +2030,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$16</f>
+              <f>'EI Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$E$2:$E$16</f>
+              <f>'EI Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -2062,12 +2062,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'EI Summary'!$A$2:$A$16</f>
+              <f>'EI Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'EI Summary'!$I$2:$I$16</f>
+              <f>'EI Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -2181,12 +2181,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$16</f>
+              <f>'MASHREQ Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$D$2:$D$16</f>
+              <f>'MASHREQ Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -2213,12 +2213,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$16</f>
+              <f>'MASHREQ Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$H$2:$H$16</f>
+              <f>'MASHREQ Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -2332,12 +2332,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$16</f>
+              <f>'MASHREQ Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$E$2:$E$16</f>
+              <f>'MASHREQ Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -2364,12 +2364,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'MASHREQ Summary'!$A$2:$A$16</f>
+              <f>'MASHREQ Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'MASHREQ Summary'!$I$2:$I$16</f>
+              <f>'MASHREQ Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -2483,12 +2483,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$16</f>
+              <f>'WIO Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$D$2:$D$16</f>
+              <f>'WIO Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -2515,12 +2515,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$16</f>
+              <f>'WIO Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$H$2:$H$16</f>
+              <f>'WIO Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -2634,12 +2634,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$16</f>
+              <f>'WIO Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$E$2:$E$16</f>
+              <f>'WIO Summary'!$E$2:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -2666,12 +2666,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'WIO Summary'!$A$2:$A$16</f>
+              <f>'WIO Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'WIO Summary'!$I$2:$I$16</f>
+              <f>'WIO Summary'!$I$2:$I$17</f>
             </numRef>
           </val>
         </ser>
@@ -2785,12 +2785,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$16</f>
+              <f>'ADCB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$D$2:$D$16</f>
+              <f>'ADCB Summary'!$D$2:$D$17</f>
             </numRef>
           </val>
         </ser>
@@ -2817,12 +2817,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ADCB Summary'!$A$2:$A$16</f>
+              <f>'ADCB Summary'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ADCB Summary'!$H$2:$H$16</f>
+              <f>'ADCB Summary'!$H$2:$H$17</f>
             </numRef>
           </val>
         </ser>
@@ -3621,7 +3621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4489,6 +4489,37 @@
         <v>3.129</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>225231</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4.689788</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>-12.968</v>
+      </c>
+      <c r="F29" t="n">
+        <v>321640</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4.73662</v>
+      </c>
+      <c r="H29" t="n">
+        <v>15</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3.021</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4501,7 +4532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7244,167 +7275,28 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>App Name</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Developer</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Average Rating</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Total Ratings</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Rating</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version Ratings Count</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Current Version</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Minimum OS</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Release Date</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.vipera.ts.starter.MashreqAE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Mashreq Bank PSC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="E2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="F2" t="n">
-        <v>4.80385</v>
-      </c>
-      <c r="G2" t="n">
-        <v>136831</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>9.16.0</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>15.1</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Free</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2010-06-30T15:18:28Z</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-04T05:13:45Z</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Finance</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Mashreq Mobile App - Invest, manage accounts, pay bills and more, securely</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7450,66 +7342,270 @@
 Dubai, UAE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-08-19</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Mashreq</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>digitalmobileonline@mashreq.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>9.18.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Mar 21, 2012</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787843891</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.7567616</v>
+      </c>
+      <c r="T17" t="n">
+        <v>144683</v>
+      </c>
+      <c r="U17" t="n">
+        <v>11162</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.mashreq.com/en/uae/neo/transparency/privacy-notice/</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9YLPmUTUHaC744bZH2BjKhrAH21uDVI2vFLjtZnS2k6hgYwXTeDvn9Fk8HTRlMDdm5TzWSsbY5zc6geNJVQDKg</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/C6so-i4Zs3Nx8O3t4ZY9n1kJlfUy8mGem0DAW8E_26GjcM7BmHjbuv5m-NKJquBKwgP10xQSA5e27iBOqW86OA</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.vipera.ts.starter.MashreqAE&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>App Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Average Rating</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Total Ratings</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Rating</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version Ratings Count</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Current Version</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Minimum OS</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="E3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4.80368</v>
-      </c>
-      <c r="G3" t="n">
-        <v>136943</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>9.17.0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="D2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="E2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.80385</v>
+      </c>
+      <c r="G2" t="n">
+        <v>136831</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>9.16.0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-18T13:56:46Z</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-08-04T05:13:45Z</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7556,65 +7652,65 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-08-20</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="E4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4.80372</v>
-      </c>
-      <c r="G4" t="n">
-        <v>137037</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="D3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="E3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.80368</v>
+      </c>
+      <c r="G3" t="n">
+        <v>136943</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7661,65 +7757,65 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="E5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4.80358</v>
-      </c>
-      <c r="G5" t="n">
-        <v>137148</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="D4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="E4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.80372</v>
+      </c>
+      <c r="G4" t="n">
+        <v>137037</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7766,65 +7862,65 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="E6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="F6" t="n">
-        <v>4.80342</v>
-      </c>
-      <c r="G6" t="n">
-        <v>137240</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="D5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="E5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.80358</v>
+      </c>
+      <c r="G5" t="n">
+        <v>137148</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7871,65 +7967,65 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="E7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="F7" t="n">
-        <v>4.80318</v>
-      </c>
-      <c r="G7" t="n">
-        <v>137331</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="D6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="E6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.80342</v>
+      </c>
+      <c r="G6" t="n">
+        <v>137240</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -7976,65 +8072,65 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="E8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4.80298</v>
-      </c>
-      <c r="G8" t="n">
-        <v>137436</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="D7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="E7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.80318</v>
+      </c>
+      <c r="G7" t="n">
+        <v>137331</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8081,65 +8177,65 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="E9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4.80291</v>
-      </c>
-      <c r="G9" t="n">
-        <v>137509</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="D8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="E8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="F8" t="n">
+        <v>4.80298</v>
+      </c>
+      <c r="G8" t="n">
+        <v>137436</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8186,65 +8282,65 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="E10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="F10" t="n">
-        <v>4.8028</v>
-      </c>
-      <c r="G10" t="n">
-        <v>137632</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="D9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="E9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4.80291</v>
+      </c>
+      <c r="G9" t="n">
+        <v>137509</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8291,65 +8387,65 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="E11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="F11" t="n">
-        <v>4.8027</v>
-      </c>
-      <c r="G11" t="n">
-        <v>137735</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="D10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="E10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.8028</v>
+      </c>
+      <c r="G10" t="n">
+        <v>137632</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8396,65 +8492,65 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="E12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="F12" t="n">
-        <v>4.80255</v>
-      </c>
-      <c r="G12" t="n">
-        <v>137879</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="D11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="E11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.8027</v>
+      </c>
+      <c r="G11" t="n">
+        <v>137735</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8501,65 +8597,65 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="E13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4.80225</v>
-      </c>
-      <c r="G13" t="n">
-        <v>138015</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="D12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="E12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="F12" t="n">
+        <v>4.80255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>137879</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8606,65 +8702,65 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-08-30</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>4.80234</v>
-      </c>
-      <c r="E14" t="n">
-        <v>138127</v>
-      </c>
-      <c r="F14" t="n">
-        <v>4.80234</v>
-      </c>
-      <c r="G14" t="n">
-        <v>138127</v>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="D13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="E13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4.80225</v>
+      </c>
+      <c r="G13" t="n">
+        <v>138015</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8711,65 +8807,65 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>4.8022</v>
-      </c>
-      <c r="E15" t="n">
-        <v>138217</v>
-      </c>
-      <c r="F15" t="n">
-        <v>4.8022</v>
-      </c>
-      <c r="G15" t="n">
-        <v>138217</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="D14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="E14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="F14" t="n">
+        <v>4.80234</v>
+      </c>
+      <c r="G14" t="n">
+        <v>138127</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>9.17.0</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-08-18T13:56:46Z</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8816,65 +8912,65 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>Mashreq UAE - Digital Banking</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Mashreq Bank PSC</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>4.80218</v>
-      </c>
-      <c r="E16" t="n">
-        <v>138299</v>
-      </c>
-      <c r="F16" t="n">
-        <v>4.80218</v>
-      </c>
-      <c r="G16" t="n">
-        <v>138299</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>9.18.0</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="D15" t="n">
+        <v>4.8022</v>
+      </c>
+      <c r="E15" t="n">
+        <v>138217</v>
+      </c>
+      <c r="F15" t="n">
+        <v>4.8022</v>
+      </c>
+      <c r="G15" t="n">
+        <v>138217</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>9.17.0</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>15.1</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>2010-06-30T15:18:28Z</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>2026-08-31T13:26:41Z</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-08-18T13:56:46Z</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>Finance</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
 Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
@@ -8921,6 +9017,216 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4.80218</v>
+      </c>
+      <c r="E16" t="n">
+        <v>138299</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.80218</v>
+      </c>
+      <c r="G16" t="n">
+        <v>138299</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>9.18.0</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-08-31T13:26:41Z</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mashreq UAE - Digital Banking</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mashreq Bank PSC</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.80216</v>
+      </c>
+      <c r="E17" t="n">
+        <v>138434</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.80216</v>
+      </c>
+      <c r="G17" t="n">
+        <v>138434</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>9.18.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2010-06-30T15:18:28Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-31T13:26:41Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Secure and convenient digital banking with Mashreq Mobile App – Smarter banking in your pocket!
+Experience the UAE’s top-rated banking app, trusted across the nation. From high-interest savings accounts and international money transfers to investment in US stocks from the UAE and family banking, discover a world of powerful financial tools at your fingertips with the award-winning, globally recognised mobile banking app.
+Open a bank account online instantly
+Open a bank account online in the UAE instantly with Mashreq - no paperwork, no waiting. Just a few taps and you're ready to bank.
+Get more value with Mashreq NEO PLUS
+• Transfer salary of AED 10,000+ or maintain an average balance of at least AED 50,000 to become eligible for exclusive Mashreq NEO PLUS benefits.
+• Mashreq NEO PLUS Saver Account: Get market-leading rates on savings — 6.25% p.a. if you transfer salary to Mashreq NEO Account OR 5% p.a. if you maintain AED 50,000+ in NEO PLUS Saver Account. Shariah-compliant Islamic products also available.
+• Fee-free everyday banking: Enjoy free ATM withdrawals worldwide, local &amp; international money transfers and chequebooks.
+Exclusive benefits with Mashreq NEO
+• Earn up to AED 9,500 cashback when you transfer your salary, refer friends, shop, remit and invest through Mashreq NEO or Mashreq Al Islami.
+• Instant digital bank account opening: Open a Mashreq NEO Account or Mashreq Al Islami Account in minutes. No paperwork required.
+• Exclusive shopping and dining offers: Enjoy fantastic discounts at your favourite outlets.
+• International money transfers: Send money to 40+ countries in a flash through Quick Remit.
+Invest in US stocks from the UAE - From just USD 1
+Explore digital wealth options — US stocks, smart portfolios, mutual funds, and more:
+• Real-time tracking.
+• Earn interest/profit on deposits.
+• Buy Mashreq Millionaire Certificates in-app.
+All-in-one banking dashboard with Mashreq Mobile App
+• Apply for credit cards, loans or financing in minutes.
+• Manage card controls, limits, PIN and spending preferences.
+• Request chequebooks, manage e-statements and update details easily.
+• Add cards to Apple Pay, Google Pay &amp; Samsung Pay digital wallets.
+Effortless transfers and payments
+• Make local and international transfers with just a few taps.
+• Transfer funds using your mobile number and email ID via Aani instant payments.
+• Recharge mobile credits and pay bills online. 
+• Cardless cash option to withdraw cash from Mashreq ATMs.
+Dedicated customer support
+Find answers fast with 24/7 Customer Care, helpful videos and our always-on chatbot Mashreq Virtual Assistant.
+Services Hub
+• All your essentials. One smart space.
+• Access over 40 services - from cardless cash withdrawal in the UAE and e-statements to letter requests and more - all within one convenient location.
+T&amp;Cs apply.
+Why Mashreq UAE Mobile App?
+Whether you're saving, spending, investing or travelling, Mashreq UAE Mobile App empowers you to do it all - securely and effortlessly.
+Download Mashreq UAE Mobile App today and start banking smarter.
+Mashreq Group HQ Building
+Plot No 3450782
+Umniyati Street (off Al Asayel Street)
+Burj Khalifa Community
+Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9028,7 +9334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9542,6 +9848,37 @@
         <v>4.494</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5828</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.6015625</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4.602</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6737</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.80793</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -9554,7 +9891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11892,6 +12229,149 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>io.wio.retail</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>See, manage, grow your money</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Wio Bank PJSC</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Wio+Bank+PJSC</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://wio.io</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>contact@wio.io</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Apr 16, 2023</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787574050</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.6015625</v>
+      </c>
+      <c r="T17" t="n">
+        <v>5828</v>
+      </c>
+      <c r="U17" t="n">
+        <v>527</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://wio.io/privacy-policy/</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/EHLNW-SlRkvzqxnM0cMAhZlltrmgETGTIjw4zn7aiIHvsypzXeSTOcodsncwMVXe2HCFxiJPQl7cJ6fWNzDWUA</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/yr3kMUS8cAp2OhipHoB6N6hZekcbFHRTc1WimtIE3NX8A0fLVrqFCBkepf76jh_pwM7rvza4oa9GukmohSyK</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=io.wio.retail&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11903,7 +12383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13145,6 +13625,84 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
+Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
+Turn your savings into earnings. Get up to 6% interest per annum when you sign up for the Wio Personal 'Salary' Plan or up to 4.75% interest per annum when you sign up for the Wio Personal 'Plus' Plan.
+One card for debit and credit. Seamlessly switch spending modes, all with the same card.
+Get rewarded for spending. Earn up to 2% cashback up to 2500 AED/month on all* credit spends with Wio Credit.
+Cashback, your way. Choose to receive it in your current account, saving space, or invest it in selected stocks.
+Travel smart, spend smarter. No foreign exchange fees + 1% cashback on your international debit transactions.
+Move money, minus the hassle. Transfer to 100+ countries with instant currency exchange at highly competitive rates.
+Instant card, instant access. Use your Wio card online immediately-add it to Apple Pay or Google Pay.
+Physical card? Order anytime.
+Virtual cards, real control. Customize your design, set spending limits, and shop securely online or in-store.
+Access 3,000+ stocks, ETFs, crypto and more-all in one secure platform.
+Crypto, simplified. Buy &amp; sell directly from your AED account-no detours, no delays.
+Be IPO-ready. Apply instantly for UAE public listings and boost your share allocation with up to 5x leverage.
+Security that works for you. Set controls on where and how you spend, backed by powerful encryption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Wio Personal</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>WIO BANK P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.80793</v>
+      </c>
+      <c r="E17" t="n">
+        <v>6737</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.80793</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6737</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1.71.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2023-07-25T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-27T04:45:31Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Open your Wio Personal account in minutes. Save, spend, borrow, manage, and invest- all in one place.
 Spend without borders, anywhere. Free multi-currency accounts in AED, USD, EUR, and GBP.
@@ -13271,7 +13829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13725,6 +14283,34 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>64308</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.212979</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-39.747</v>
+      </c>
+      <c r="F17" t="n">
+        <v>113008</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -13737,7 +14323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16075,6 +16661,149 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.adcb.bank</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips with the ADCB Mobile App</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>http://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Mar 31, 2013</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1779603200</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.212979</v>
+      </c>
+      <c r="T17" t="n">
+        <v>64308</v>
+      </c>
+      <c r="U17" t="n">
+        <v>15245</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/le83ha0sIaB5qSpbmYUawJInroj0U7hqj61xuLKiqcOLBAbwY8aAQg7eq2447aDDf7Y6q8Pfuw3TY31q3Q7F</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8Nj1GiTeIRhiJ85lKBKal8z8d5wF3ibyhBxwJzZAK9aK0niSrau_Mzq7TzRbFb5Kjm8Veh-PA7aX8MkAo-6h</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.bank&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16086,7 +16815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17362,6 +18091,85 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ADCB</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="E17" t="n">
+        <v>113008</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.68156</v>
+      </c>
+      <c r="G17" t="n">
+        <v>113008</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>21.5.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>12.2</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2012-10-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-06-05T16:38:30Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Experience more power at your fingertips.
+Experience the new and improved mobile banking app from ADCB. Enjoy seamless banking on-the-go with the enhanced features combined with an intuitive and user-friendly visual experience.
+More power at your fingertips
+- A simplified 'Payments and Transfers' section where you can view your beneficiaries and registered billers all in one screen
+- Search Payees and Transaction History by name, amount and much more
+- Dual language option in Arabic and English
+Plus, you can continue to enjoy these services
+- Balance Preview
+- Bill Payment
+- Funds Transfer
+- Locate ADCB ATM and Branches
+If you are a new ADCB Mobile App user or if you are using the app on a new device, register with the following steps:
+- Download and launch the ADCB Mobile App
+- When prompted, enter your ADCB Credit Card/Debit Card Number and PIN; enter the activation key that is sent to your registered mobile number
+- Alternatively, you can enter your ADCB Customer ID and activation key which you can obtain through our Personal Internet Banking or the 24/7 Contact Centre
+If you are an existing user, you will be prompted to enter your existing ADCB Mobile App password for authentication and biometric re-enrollment (handset dependent).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17373,7 +18181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE28"/>
+  <dimension ref="A1:AE29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21238,6 +22046,142 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>com.emiratesnbd.android</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Emirates NBD Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Elevate your mobile banking by innovations with ENBD X; finance your needs, get 150+ instant services and invest with various digital wealth options.
+With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services.
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X.
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app.
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey.
+Download the app today to enjoy the numerous features and benefits that Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Emirates NBD</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>7061249469913377530</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>http://www.emiratesnbd.com/en/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>tech@emiratesnbd.com</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Dec 12, 2021</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>1787789548</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q29" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R29" t="n">
+        <v>4.689788</v>
+      </c>
+      <c r="T29" t="n">
+        <v>225231</v>
+      </c>
+      <c r="U29" t="n">
+        <v>17225</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W29" t="b">
+        <v>1</v>
+      </c>
+      <c r="X29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z29" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA29" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>https://www.emiratesnbd.com/en/terms-conditions/mobile-privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/nGu208TZJ8mlMHWrbhtE6399F7BOz1bKyrA4i_zxpchKpSdlrN5qfvaUMvXe8n2UPXYxTL3a5QsU_Md-PoXBZA</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/CejgWNSjMgSJeRK1Ivl-l4tXVRGNV7ZR-caLbNSHkm5KQeRUL1pxlYWVM3j84hC_JGAp3YypFZrLbySQapcQXA</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesnbd.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21339,7 +22283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21853,6 +22797,37 @@
         <v>4.699</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>75300</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.670211</v>
+      </c>
+      <c r="D17" t="n">
+        <v>270</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.886</v>
+      </c>
+      <c r="F17" t="n">
+        <v>77016</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.47713</v>
+      </c>
+      <c r="H17" t="n">
+        <v>321</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.652</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -21865,7 +22840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24248,6 +25223,152 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.adcb.nexgen</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ADCB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalized over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Commercial+Bank</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>riskandcontrolit@adcb.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Apr 20, 2026</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1788059707</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.670211</v>
+      </c>
+      <c r="T17" t="n">
+        <v>75300</v>
+      </c>
+      <c r="U17" t="n">
+        <v>4966</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.adcb.com/mib/Privacy-Policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/8a4DBrLNpCk2XKnynAoQehCM2c6NkywlCNyVIXa7QfKAJX4g7I6Meew9zSrjMapeCbGL8VzQRxbCUXGMYWH1Luo</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/9_mP55V12dDRLxjYHqEt4w74qpIhuOF82hYTZRx8KpL8Nipnb62wbo9auj0L7KTvZ9BsliIqogav5cHTfyABQA</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adcb.nexgen&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -24259,7 +25380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25543,6 +26664,87 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
+The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
+Designed to simplify the way you manage your finances, the app brings together intelligent features, seamless navigation, and secure access, all in one place.
+AI-powered smart banking
+Experience smarter banking with advanced AI that provides intuitive prompts and helps you complete tasks quickly across a wide range of services.
+Faster, more seamless experience
+View and manage your accounts, cards, loans, and services in one place, with improved speed, smoother navigation, and quicker access to what matters most.
+Intuitive end-to-end journeys
+Every journey has been redesigned to be simpler, clearer, and easier to complete, from everyday transactions to more advanced banking needs.
+All-in-one banking
+Open accounts, apply for products, manage your cards, and build your investment portfolio, all within one secure app.
+Investment and trading
+Access global markets directly from the app and trade US equities, ETFs, and cryptocurrencies with real-time market data.
+Secure and convenient access
+Sign in quickly using biometrics or UAE Pass, with enhanced security built into every interaction.
+This is just the beginning.
+The ADCB Mobile Banking App will continue to evolve with every update, becoming more intuitive, more helpful, and more personalised over time.
+A smarter way to bank, built around your daily life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ADCB.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Commercial Bank</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.47713</v>
+      </c>
+      <c r="E17" t="n">
+        <v>77016</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.47713</v>
+      </c>
+      <c r="G17" t="n">
+        <v>77016</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-04-15T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-31T15:36:25Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Welcome to a new era of banking. Powered by AI. Shaped by you.
 The new ADCB Mobile Banking App is powered by advanced AI and built with a next-generation digital experience, making banking faster, more intuitive, and seamlessly connected to your everyday needs.
@@ -25672,7 +26874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26186,6 +27388,37 @@
         <v>4.614</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>45463</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.6379604</v>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5.762</v>
+      </c>
+      <c r="F17" t="n">
+        <v>252708</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.70119</v>
+      </c>
+      <c r="H17" t="n">
+        <v>76</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.97</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -26198,7 +27431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28746,6 +29979,163 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.adib.mobile</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Manage your money on the go. Mobile banking as it should be!</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>The all-new ADIB Mobile Banking gives you the freedom to manage your money on the go. View all your accounts at a glance, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more! +  +
+Features include: 
+             A timeline of all your account transactions
+             Transaction detail with a single tap
+             Ability to temporarily block your card &amp; request for card replacements
+             Get personal finance from the comfort of your home (if you qualify)
+             Option to personalize your app with images for accounts
+             One place for all your payments
+             Update Emirates ID, Passport, mobile number and email
+             View your personal, identification and contact details
+             Transfer money from your ADIB Visa or MasterCard to your account
+             Pay bills with your Visa / MasterCard
+             Open a new account
+             View exchange rates for your foreign currency accounts
+             Location of all ADIB Branches &amp; ATMs
+             Register for phone banking, SMS banking and e-statements
+             Change your Phone Banking ePIN
+             View your Financing and Card transaction details
+             Search transactions by entering keywords
+             View pending transactions
+             Apply for an ADIB service (Certificates, Chequebooks, etc.)
+             Improved look &amp; feel
+             Donate to Red Crescent Sukuk directly within the app  
+             Push notifications – Get offers that you like
+             Request new products / services directly within the app
+             View your ADIB Covered card benefits
+             Log in the app with your Fingerprint</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Abu Dhabi Islamic Bank</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Abu+Dhabi+Islamic+Bank</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>http://www.adib.ae</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>onlinehelp@adib.ae</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Oct 16, 2016</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787072896</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.6379604</v>
+      </c>
+      <c r="T17" t="n">
+        <v>45463</v>
+      </c>
+      <c r="U17" t="n">
+        <v>15064</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.adib.ae/en/pages/privacy_policy.aspx</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/rKU3NCf_sJi0Q4XDMcZnblIUBY3sHcb6OhKtsD-cka7ZRI4ysSioTsL7thYCb9LJzANJK5M1EIin2v_4DWy_</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/Mhwlq9jGoLa1Yhf7YAkoEFmLXwGLI79urScU2tik1GzE44O92tjnXMsxjqwl01g-LHo-Ta3xO3ok1Emn0B4nUw</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.adib.mobile&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -28757,7 +30147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30139,6 +31529,94 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
+Features include: 
+·  A timeline of all your account transactions
+·  Transaction detail with a single tap
+·  Enhanced security - Login with Touch ID or Face ID
+·  Ability to temporarily block your card &amp; request for card replacements
+·  Get personal finance from the comfort of your home (if you qualify)
+·  Option to personalize your app with images for accounts
+·  One place for all your payments
+·  Update Emirates ID, Passport, mobile number and email
+·  View your personal, identification and contact details
+·  Transfer money from your ADIB Visa or MasterCard to your account
+·  Pay bills with your Visa / MasterCard
+·  Open a new account
+·  View exchange rates for your foreign currency accounts
+·  Location of all ADIB Branches &amp; ATMs
+·  Register for phone banking, SMS banking and e-statements
+·  Change your Phone Banking ePIN
+·  View your Financing and Card transaction details
+·  Search transactions by entering keywords
+·  View pending transactions
+·  Apply for an ADIB service (Certificates, Chequebooks, etc.)
+·  Push notifications – Get offers that you like
+·  Request new products / services directly within the app
+·  View your ADIB Covered card benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ADIB Mobile Banking</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ABU DHABI ISLAMIC BANK</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.70119</v>
+      </c>
+      <c r="E17" t="n">
+        <v>252708</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.70119</v>
+      </c>
+      <c r="G17" t="n">
+        <v>252708</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>8.8.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>13.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2016-09-29T11:47:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-18T17:03:50Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>The ADIB Mobile Banking app gives you the freedom to manage your money on the go. View all your accounts at a glance, pay your bills, send money to your family &amp; friends, pay your bills, recharge your phone &amp; Salik credit, apply for financing and much more!
 Features include: 
@@ -30275,7 +31753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30789,6 +32267,37 @@
         <v>4.938</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>43955</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.312464</v>
+      </c>
+      <c r="D17" t="n">
+        <v>27</v>
+      </c>
+      <c r="E17" t="n">
+        <v>7.216</v>
+      </c>
+      <c r="F17" t="n">
+        <v>111953</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.63501</v>
+      </c>
+      <c r="H17" t="n">
+        <v>85</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.872</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -30801,7 +32310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32782,6 +34291,76 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ENBD X</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>EMIRATES NBD Bank (P.J.S.C)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>4.73662</v>
+      </c>
+      <c r="E29" t="n">
+        <v>321640</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.73662</v>
+      </c>
+      <c r="G29" t="n">
+        <v>321640</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2021-12-19T08:00:00Z</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:44:56Z</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>With ENBD X, a new standard of excellence, embark on a groundbreaking journey to mobile banking on your phone. Seamlessly navigate through all your Emirates NBD products to gain control of your finances. This cutting-edge app empowers you to securely manage your accounts and cards with the assurance from Emirates NBD to bring you best in class banking products and services. 
+Emirates NBD, known for its commitment to innovation, ensures your financial wellbeing and security with ENBD X. 
+Access over 150+ services, with majority of them being processed instantly on the app with no extra steps. Lock and unlock your Emirates NBD card effortlessly, reset your card PIN, request statements, letters with just a few taps, and set precise spending and withdrawal limits to match your financial preferences. See the historical information about your transactions on your accounts, cards and loans. Moreover, you can open an investment portfolio instantly and start trading in Global and Local Equities. You can find best of deals, offers and benefits of banking with Emirates NBD with the ease and convenience of the ENBD X mobile app. 
+ENBD X, proudly brought to you by Emirates NBD, not only simplifies your daily digital banking but also offers lightning-fast international money transfer feature to multiple destinations with DirectRemit. Additionally, managing your finances is a breeze, as you can conveniently pay your bills or top up your mobile phone with Emirates NBD's secure and user-friendly app.
+Embrace banking like never before with Emirates NBD's ENBD X app – your trusted companion for a seamless, secure, and efficient financial journey. 
+Download the app today to enjoy the numerous features and benefits Emirates NBD has tailored exclusively for you.
+Privacy Policy URL: https://www.emiratesnbd.com/en/data-privacy-notice/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32793,7 +34372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -35266,6 +36845,158 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.fab.personalbanking</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Spend, save and stay on top of your everyday banking from just about anywhere.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>FIRST+ABU+DHABI+BANK</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/contact-us</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>atyourservice@bankfab.com</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>3.7.68</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Dec 3, 2018</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787322295</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.312464</v>
+      </c>
+      <c r="T17" t="n">
+        <v>43955</v>
+      </c>
+      <c r="U17" t="n">
+        <v>12415</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.bankfab.com/en-ae/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/HVvcbMD1E5pSDM-EGX_miuChGLwygensVGuPhNI1PwnX8WmgIo9R6GimqoY6M2aJqxkrYrZn6DsrwKxZeJb1qA</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/AeCnxbQPkvIP6r101HfPcMoxOkd4P1xlAczLsC_8Eva_-ahkJngHtPOD83yGu5UUJEUemc8WDVRuJNzu_nF-0lI</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.fab.personalbanking&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35277,7 +37008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -36645,6 +38376,93 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>Let’s bring the bank to YOU! 
+The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
+DOWNLOAD. REGISTER. DONE!
+If you’re a FAB customer or using the app on a new device, here’s how you can get started once you download the app:
+•	Tap ‘Already a customer’ and enter your credit or debit card number or customer number
+•	Tap and scan your Emirates ID
+•	Do the face scan as prompted – to ensure that only you have access to your account
+•	You’re done! Now you can start banking anywhere, anytime.   
+NEW CUSTOMER? NO PROBLEM!
+Start your journey with FAB right from your living room. Simply download the app and open an account, get a credit card or get approved for a personal loan – without stepping into a branch. You only need an Emirates ID. 
+YOUR MONEY. YOUR WAY.
+We know you value your time, so we’ve made sure you can do a whole lot of your banking, whenever you want. Here are some of things you can do:
+•	View your balance and e-statements
+•	Activate your card
+•	Pay your utility bills
+•	Get an Easy Payment Plan 
+•	Sign up for Islamic accounts
+•	Earn and redeem FAB Rewards
+•	Start an iSave and enjoy a higher rate of interest
+•	Upload your account documents – passport, visa, Emirates ID
+•	Login with Fingerprint or Face ID
+•	Locate your nearest FAB branch or ATM
+•	Enjoy free and instant transfers to India, Pakistan, Sri Lanka and Philippines 
+•	Enjoy exciting offers and exclusive discounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FAB Mobile</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FIRST ABU DHABI BANK PJSC</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.63501</v>
+      </c>
+      <c r="E17" t="n">
+        <v>111953</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.63501</v>
+      </c>
+      <c r="G17" t="n">
+        <v>111953</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2.0.93</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2018-12-04T03:28:01Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-23T16:15:07Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Let’s bring the bank to YOU! 
 The FAB Mobile app puts the power of the bank in your hand. Spend, save and stay on top of your everyday banking from just about anywhere. 
@@ -36780,7 +38598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37255,6 +39073,34 @@
         <v>3.961</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>46157</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.480045</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>33723</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.635</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.118</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -37267,7 +39113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -39620,6 +41466,150 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.rak</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Digital with a human touch</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>RAKBANK</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://rakbank.ae/wps/portal/info/digital-banking?WT.ac=Digital_Banking_HP_banner</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>marketing@rakbank.ae</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>350.60.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Aug 2, 2011</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787754965</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1,000,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.480045</v>
+      </c>
+      <c r="T17" t="n">
+        <v>46157</v>
+      </c>
+      <c r="U17" t="n">
+        <v>3261</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.rakbank.ae/en/privacy-policy</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/z6rXT0eBpe4SBiVyR_HrIwcRZz9m8lHRHtGW_NZ4UzERlfOk59lDrqC0r43BRltbYhGlVCBpTGGe54pwRkD6Yw</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/L0KLPUHnfeutuurS8hYI1muO9OiwDzN9Yo7j9Ca2Dfo3ZIaXuep8KYVVLOBrvLCfzMHHexvPrOjL2MU-LEoWFw</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.rak&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -39631,7 +41621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -40887,6 +42877,85 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>Our app brings you a simple yet secure way to manage, move and grow your money.
+YOUR MONEY ON YOUR TERMS
+- Get a clearer, more intuitive view of your finances from the moment you log in
+- Bank your way and enjoy a full experience in English or Arabic
+- Make your money work for you with gold, silver, crypto and other investments
+- Full control over cards, limits and repayments
+PAYMENTS MADE SIMPLE
+- One place for every payment
+- Send money across the UAE and abroad in a few taps
+- Pay all your due bills in one go
+- Repeat payments: set once, sorted forever
+- Send cash to contacts instantly
+- Get cardless withdrawals from any of our ATMs with Mobile cash
+- Donate to causes you care about, straight from the app
+MEET RAI, YOUR DIGITAL ASSISTANT
+Stuck? Just ask Rai. Instant answers, zero hunting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Rakbank</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>National Bank of Ras Al Khaimah</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.635</v>
+      </c>
+      <c r="E17" t="n">
+        <v>33723</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.635</v>
+      </c>
+      <c r="G17" t="n">
+        <v>33723</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>15.1</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2011-03-31T18:05:11Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-27T14:25:32Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Our app brings you a simple yet secure way to manage, move and grow your money.
 YOUR MONEY ON YOUR TERMS
@@ -41110,7 +43179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41597,6 +43666,34 @@
         <v>4.717</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>73826</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.6703873</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>113679</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.71734</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3.865</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -41609,7 +43706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -43722,6 +45819,134 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>com.emiratesislamic.android</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>The all new EI Bank P.J.S.C Mobile App</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>We've lined up some exciting updates just in time for holiday season:
+• Now you can find the Emirates Islamic Branches &amp; ATM location with EI +.
+• Sending money to other  Emirates Islamic, Emirates NBD and Liv accounts is now easier with entering account number, only.
+• Update your Prepaid card nickname instantly.
+Thank you for banking with Emirates Islamic.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>EMIRATES ISLAMIC BANK (PJSC)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>EMIRATES+ISLAMIC+BANK+(PJSC)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Apps@emiratesislamic.ae</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Apr 7, 2022</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1787790542</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>500,000+</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>500000</v>
+      </c>
+      <c r="R17" t="n">
+        <v>4.6703873</v>
+      </c>
+      <c r="T17" t="n">
+        <v>73826</v>
+      </c>
+      <c r="U17" t="n">
+        <v>5922</v>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>PEGI 3</t>
+        </is>
+      </c>
+      <c r="W17" t="b">
+        <v>1</v>
+      </c>
+      <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>AED</t>
+        </is>
+      </c>
+      <c r="Z17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>https://www.emiratesislamic.ae/en/data-privacy-notice</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/LF1qBFjyS9vVxWTRdGHMIE9rOB3-5b32Cchhd51gv4QnRkjkdNFtqk8tUo2AerXfeA_mU3_P2nBQf1J4QG4z</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>https://play-lh.googleusercontent.com/InV3dloiiTmXjQE1W8-vJJdbZc2rUAPtCFPWAnIpt0v0vqePJP0dArg_DK8zqWFl6BldvTlSGkn3A5FgOj9yFkE</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>https://play.google.com/store/apps/details?id=com.emiratesislamic.android&amp;hl=en&amp;gl=ae</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -43733,7 +45958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -44779,6 +47004,70 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EI +</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Emirates Islamic Bank P.J.S.C</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>4.71734</v>
+      </c>
+      <c r="E17" t="n">
+        <v>113679</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.71734</v>
+      </c>
+      <c r="G17" t="n">
+        <v>113679</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>26.8.10</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2022-04-18T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-08-27T16:42:57Z</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Emirates Islamic's newest mobile banking offering brings the latest in technology, and enhanced user experience to our existing and new clients.</t>
         </is>
@@ -44891,7 +47180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45405,6 +47694,37 @@
         <v>4.768</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>144683</v>
+      </c>
+      <c r="C17" t="n">
+        <v>4.7567616</v>
+      </c>
+      <c r="D17" t="n">
+        <v>185</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3.921</v>
+      </c>
+      <c r="F17" t="n">
+        <v>138434</v>
+      </c>
+      <c r="G17" t="n">
+        <v>4.80216</v>
+      </c>
+      <c r="H17" t="n">
+        <v>135</v>
+      </c>
+      <c r="I17" t="n">
+        <v>4.782</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>